<commit_message>
Edit PDS and Change Dashboard
</commit_message>
<xml_diff>
--- a/public/pds.xlsx
+++ b/public/pds.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cenro\Deniel\System\rsp-hr-tagum-cityhall\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9D6E79A-1318-4407-9240-412ADD37B84B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91D909C6-055F-45E3-8D39-0189505429EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="795" yWindow="2490" windowWidth="28800" windowHeight="17145" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Personal Information" sheetId="16" r:id="rId1"/>
@@ -1615,7 +1615,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="345">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="346">
   <si>
     <t xml:space="preserve">        </t>
   </si>
@@ -2702,6 +2702,9 @@
   </si>
   <si>
     <t xml:space="preserve">     PDS_RSP_OFFICIAL_2026                                                                                                                                                       </t>
+  </si>
+  <si>
+    <t>ETHNIC GROUP</t>
   </si>
 </sst>
 </file>
@@ -3738,7 +3741,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="35" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="502">
+  <cellXfs count="503">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="166" fontId="18" fillId="0" borderId="47" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
@@ -4367,12 +4370,19 @@
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
     <xf numFmtId="49" fontId="22" fillId="3" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="28" fillId="3" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="35" fillId="0" borderId="39" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -5144,18 +5154,6 @@
     </xf>
     <xf numFmtId="49" fontId="7" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
@@ -5335,6 +5333,18 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -5418,10 +5428,6 @@
     <xf numFmtId="49" fontId="7" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" wrapText="1"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection hidden="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -10867,20 +10873,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="2.25" customHeight="1" thickBot="1">
-      <c r="A1" s="227"/>
-      <c r="B1" s="228"/>
-      <c r="C1" s="228"/>
-      <c r="D1" s="228"/>
-      <c r="E1" s="228"/>
-      <c r="F1" s="228"/>
-      <c r="G1" s="228"/>
-      <c r="H1" s="228"/>
-      <c r="I1" s="228"/>
-      <c r="J1" s="228"/>
-      <c r="K1" s="228"/>
-      <c r="L1" s="228"/>
-      <c r="M1" s="228"/>
-      <c r="N1" s="229"/>
+      <c r="A1" s="229"/>
+      <c r="B1" s="230"/>
+      <c r="C1" s="230"/>
+      <c r="D1" s="230"/>
+      <c r="E1" s="230"/>
+      <c r="F1" s="230"/>
+      <c r="G1" s="230"/>
+      <c r="H1" s="230"/>
+      <c r="I1" s="230"/>
+      <c r="J1" s="230"/>
+      <c r="K1" s="230"/>
+      <c r="L1" s="230"/>
+      <c r="M1" s="230"/>
+      <c r="N1" s="231"/>
     </row>
     <row r="2" spans="1:22" ht="11.25" customHeight="1">
       <c r="A2" s="40"/>
@@ -10899,7 +10905,7 @@
       </c>
       <c r="M2" s="41"/>
       <c r="N2" s="42"/>
-      <c r="O2" s="501" t="s">
+      <c r="O2" s="194" t="s">
         <v>344</v>
       </c>
       <c r="Q2" s="52" t="s">
@@ -10910,69 +10916,69 @@
       </c>
     </row>
     <row r="3" spans="1:22" ht="41.25" customHeight="1">
-      <c r="A3" s="233" t="s">
+      <c r="A3" s="235" t="s">
         <v>343</v>
       </c>
-      <c r="B3" s="234"/>
-      <c r="C3" s="234"/>
-      <c r="D3" s="234"/>
-      <c r="E3" s="234"/>
-      <c r="F3" s="234"/>
-      <c r="G3" s="234"/>
-      <c r="H3" s="234"/>
-      <c r="I3" s="234"/>
-      <c r="J3" s="234"/>
-      <c r="K3" s="234"/>
-      <c r="L3" s="234"/>
-      <c r="M3" s="234"/>
-      <c r="N3" s="235"/>
-      <c r="R3" s="266"/>
-      <c r="S3" s="267"/>
-      <c r="T3" s="267"/>
-      <c r="U3" s="267"/>
-      <c r="V3" s="268"/>
+      <c r="B3" s="236"/>
+      <c r="C3" s="236"/>
+      <c r="D3" s="236"/>
+      <c r="E3" s="236"/>
+      <c r="F3" s="236"/>
+      <c r="G3" s="236"/>
+      <c r="H3" s="236"/>
+      <c r="I3" s="236"/>
+      <c r="J3" s="236"/>
+      <c r="K3" s="236"/>
+      <c r="L3" s="236"/>
+      <c r="M3" s="236"/>
+      <c r="N3" s="237"/>
+      <c r="R3" s="268"/>
+      <c r="S3" s="269"/>
+      <c r="T3" s="269"/>
+      <c r="U3" s="269"/>
+      <c r="V3" s="270"/>
     </row>
     <row r="4" spans="1:22" ht="21.75" customHeight="1">
-      <c r="A4" s="233"/>
-      <c r="B4" s="234"/>
-      <c r="C4" s="234"/>
-      <c r="D4" s="234"/>
-      <c r="E4" s="234"/>
-      <c r="F4" s="234"/>
-      <c r="G4" s="234"/>
-      <c r="H4" s="234"/>
-      <c r="I4" s="234"/>
-      <c r="J4" s="234"/>
-      <c r="K4" s="234"/>
-      <c r="L4" s="234"/>
-      <c r="M4" s="234"/>
-      <c r="N4" s="235"/>
-      <c r="R4" s="269"/>
-      <c r="S4" s="270"/>
-      <c r="T4" s="270"/>
-      <c r="U4" s="270"/>
-      <c r="V4" s="271"/>
+      <c r="A4" s="235"/>
+      <c r="B4" s="236"/>
+      <c r="C4" s="236"/>
+      <c r="D4" s="236"/>
+      <c r="E4" s="236"/>
+      <c r="F4" s="236"/>
+      <c r="G4" s="236"/>
+      <c r="H4" s="236"/>
+      <c r="I4" s="236"/>
+      <c r="J4" s="236"/>
+      <c r="K4" s="236"/>
+      <c r="L4" s="236"/>
+      <c r="M4" s="236"/>
+      <c r="N4" s="237"/>
+      <c r="R4" s="271"/>
+      <c r="S4" s="272"/>
+      <c r="T4" s="272"/>
+      <c r="U4" s="272"/>
+      <c r="V4" s="273"/>
     </row>
     <row r="5" spans="1:22" ht="11.25" customHeight="1">
-      <c r="A5" s="233"/>
-      <c r="B5" s="234"/>
-      <c r="C5" s="234"/>
-      <c r="D5" s="234"/>
-      <c r="E5" s="234"/>
-      <c r="F5" s="234"/>
-      <c r="G5" s="234"/>
-      <c r="H5" s="234"/>
-      <c r="I5" s="234"/>
-      <c r="J5" s="234"/>
-      <c r="K5" s="234"/>
-      <c r="L5" s="234"/>
-      <c r="M5" s="234"/>
-      <c r="N5" s="235"/>
-      <c r="R5" s="269"/>
-      <c r="S5" s="270"/>
-      <c r="T5" s="270"/>
-      <c r="U5" s="270"/>
-      <c r="V5" s="271"/>
+      <c r="A5" s="235"/>
+      <c r="B5" s="236"/>
+      <c r="C5" s="236"/>
+      <c r="D5" s="236"/>
+      <c r="E5" s="236"/>
+      <c r="F5" s="236"/>
+      <c r="G5" s="236"/>
+      <c r="H5" s="236"/>
+      <c r="I5" s="236"/>
+      <c r="J5" s="236"/>
+      <c r="K5" s="236"/>
+      <c r="L5" s="236"/>
+      <c r="M5" s="236"/>
+      <c r="N5" s="237"/>
+      <c r="R5" s="271"/>
+      <c r="S5" s="272"/>
+      <c r="T5" s="272"/>
+      <c r="U5" s="272"/>
+      <c r="V5" s="273"/>
     </row>
     <row r="6" spans="1:22" ht="36.75" hidden="1" customHeight="1">
       <c r="A6" s="43"/>
@@ -10989,11 +10995,11 @@
       <c r="L6" s="45"/>
       <c r="M6" s="45"/>
       <c r="N6" s="46"/>
-      <c r="R6" s="269"/>
-      <c r="S6" s="270"/>
-      <c r="T6" s="270"/>
-      <c r="U6" s="270"/>
-      <c r="V6" s="271"/>
+      <c r="R6" s="271"/>
+      <c r="S6" s="272"/>
+      <c r="T6" s="272"/>
+      <c r="U6" s="272"/>
+      <c r="V6" s="273"/>
     </row>
     <row r="7" spans="1:22" s="53" customFormat="1" ht="12.75" customHeight="1" thickBot="1">
       <c r="A7" s="47" t="s">
@@ -11011,197 +11017,197 @@
       <c r="K7" s="51" t="s">
         <v>4</v>
       </c>
-      <c r="L7" s="230" t="s">
+      <c r="L7" s="232" t="s">
         <v>5</v>
       </c>
-      <c r="M7" s="231"/>
-      <c r="N7" s="232"/>
-      <c r="R7" s="269"/>
-      <c r="S7" s="270"/>
-      <c r="T7" s="270"/>
-      <c r="U7" s="270"/>
-      <c r="V7" s="271"/>
+      <c r="M7" s="233"/>
+      <c r="N7" s="234"/>
+      <c r="R7" s="271"/>
+      <c r="S7" s="272"/>
+      <c r="T7" s="272"/>
+      <c r="U7" s="272"/>
+      <c r="V7" s="273"/>
     </row>
     <row r="8" spans="1:22" ht="2.25" customHeight="1" thickBot="1">
       <c r="A8" s="54"/>
       <c r="N8" s="55"/>
-      <c r="R8" s="269"/>
-      <c r="S8" s="270"/>
-      <c r="T8" s="270"/>
-      <c r="U8" s="270"/>
-      <c r="V8" s="271"/>
+      <c r="R8" s="271"/>
+      <c r="S8" s="272"/>
+      <c r="T8" s="272"/>
+      <c r="U8" s="272"/>
+      <c r="V8" s="273"/>
     </row>
     <row r="9" spans="1:22" ht="16.5" customHeight="1" thickBot="1">
-      <c r="A9" s="280" t="s">
+      <c r="A9" s="282" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="281"/>
-      <c r="C9" s="281"/>
-      <c r="D9" s="281"/>
-      <c r="E9" s="281"/>
-      <c r="F9" s="281"/>
-      <c r="G9" s="281"/>
-      <c r="H9" s="281"/>
-      <c r="I9" s="281"/>
-      <c r="J9" s="281"/>
-      <c r="K9" s="281"/>
-      <c r="L9" s="281"/>
-      <c r="M9" s="281"/>
-      <c r="N9" s="282"/>
-      <c r="R9" s="269"/>
-      <c r="S9" s="270"/>
-      <c r="T9" s="270"/>
-      <c r="U9" s="270"/>
-      <c r="V9" s="271"/>
+      <c r="B9" s="283"/>
+      <c r="C9" s="283"/>
+      <c r="D9" s="283"/>
+      <c r="E9" s="283"/>
+      <c r="F9" s="283"/>
+      <c r="G9" s="283"/>
+      <c r="H9" s="283"/>
+      <c r="I9" s="283"/>
+      <c r="J9" s="283"/>
+      <c r="K9" s="283"/>
+      <c r="L9" s="283"/>
+      <c r="M9" s="283"/>
+      <c r="N9" s="284"/>
+      <c r="R9" s="271"/>
+      <c r="S9" s="272"/>
+      <c r="T9" s="272"/>
+      <c r="U9" s="272"/>
+      <c r="V9" s="273"/>
     </row>
     <row r="10" spans="1:22" ht="22.5" customHeight="1">
       <c r="A10" s="56">
         <v>2</v>
       </c>
-      <c r="B10" s="252" t="s">
+      <c r="B10" s="254" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="240"/>
-      <c r="D10" s="283"/>
-      <c r="E10" s="283"/>
-      <c r="F10" s="283"/>
-      <c r="G10" s="283"/>
-      <c r="H10" s="283"/>
-      <c r="I10" s="283"/>
-      <c r="J10" s="283"/>
-      <c r="K10" s="283"/>
-      <c r="L10" s="283"/>
-      <c r="M10" s="283"/>
-      <c r="N10" s="284"/>
+      <c r="C10" s="242"/>
+      <c r="D10" s="285"/>
+      <c r="E10" s="285"/>
+      <c r="F10" s="285"/>
+      <c r="G10" s="285"/>
+      <c r="H10" s="285"/>
+      <c r="I10" s="285"/>
+      <c r="J10" s="285"/>
+      <c r="K10" s="285"/>
+      <c r="L10" s="285"/>
+      <c r="M10" s="285"/>
+      <c r="N10" s="286"/>
       <c r="P10" s="57" t="s">
         <v>8</v>
       </c>
-      <c r="R10" s="269"/>
-      <c r="S10" s="270"/>
-      <c r="T10" s="270"/>
-      <c r="U10" s="270"/>
-      <c r="V10" s="271"/>
+      <c r="R10" s="271"/>
+      <c r="S10" s="272"/>
+      <c r="T10" s="272"/>
+      <c r="U10" s="272"/>
+      <c r="V10" s="273"/>
     </row>
     <row r="11" spans="1:22" ht="22.5" customHeight="1">
       <c r="A11" s="58"/>
-      <c r="B11" s="253" t="s">
+      <c r="B11" s="255" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="254"/>
-      <c r="D11" s="285"/>
-      <c r="E11" s="286"/>
-      <c r="F11" s="286"/>
-      <c r="G11" s="286"/>
-      <c r="H11" s="287"/>
-      <c r="I11" s="288" t="s">
+      <c r="C11" s="256"/>
+      <c r="D11" s="287"/>
+      <c r="E11" s="288"/>
+      <c r="F11" s="288"/>
+      <c r="G11" s="288"/>
+      <c r="H11" s="289"/>
+      <c r="I11" s="290" t="s">
         <v>10</v>
       </c>
-      <c r="J11" s="289"/>
-      <c r="K11" s="289"/>
-      <c r="L11" s="290"/>
-      <c r="M11" s="291"/>
-      <c r="N11" s="292"/>
+      <c r="J11" s="291"/>
+      <c r="K11" s="291"/>
+      <c r="L11" s="292"/>
+      <c r="M11" s="293"/>
+      <c r="N11" s="294"/>
       <c r="P11" s="60" t="s">
         <v>11</v>
       </c>
       <c r="Q11" s="61" t="s">
         <v>12</v>
       </c>
-      <c r="R11" s="269"/>
-      <c r="S11" s="270"/>
-      <c r="T11" s="270"/>
-      <c r="U11" s="270"/>
-      <c r="V11" s="271"/>
+      <c r="R11" s="271"/>
+      <c r="S11" s="272"/>
+      <c r="T11" s="272"/>
+      <c r="U11" s="272"/>
+      <c r="V11" s="273"/>
     </row>
     <row r="12" spans="1:22" ht="21.75" customHeight="1" thickBot="1">
       <c r="A12" s="62"/>
-      <c r="B12" s="275" t="s">
+      <c r="B12" s="277" t="s">
         <v>13</v>
       </c>
-      <c r="C12" s="276"/>
-      <c r="D12" s="277"/>
-      <c r="E12" s="278"/>
-      <c r="F12" s="278"/>
-      <c r="G12" s="278" t="b">
+      <c r="C12" s="278"/>
+      <c r="D12" s="279"/>
+      <c r="E12" s="280"/>
+      <c r="F12" s="280"/>
+      <c r="G12" s="280" t="b">
         <v>0</v>
       </c>
-      <c r="H12" s="278"/>
-      <c r="I12" s="278" t="b">
+      <c r="H12" s="280"/>
+      <c r="I12" s="280" t="b">
         <v>1</v>
       </c>
-      <c r="J12" s="278"/>
-      <c r="K12" s="278"/>
-      <c r="L12" s="278"/>
-      <c r="M12" s="278"/>
-      <c r="N12" s="279"/>
+      <c r="J12" s="280"/>
+      <c r="K12" s="280"/>
+      <c r="L12" s="280"/>
+      <c r="M12" s="280"/>
+      <c r="N12" s="281"/>
       <c r="P12" s="60" t="s">
         <v>14</v>
       </c>
       <c r="Q12" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="R12" s="269"/>
-      <c r="S12" s="270"/>
-      <c r="T12" s="270"/>
-      <c r="U12" s="270"/>
-      <c r="V12" s="271"/>
+      <c r="R12" s="271"/>
+      <c r="S12" s="272"/>
+      <c r="T12" s="272"/>
+      <c r="U12" s="272"/>
+      <c r="V12" s="273"/>
     </row>
     <row r="13" spans="1:22" ht="24" customHeight="1">
       <c r="A13" s="63">
         <v>3</v>
       </c>
-      <c r="B13" s="239" t="s">
+      <c r="B13" s="241" t="s">
         <v>329</v>
       </c>
-      <c r="C13" s="240"/>
-      <c r="D13" s="248"/>
-      <c r="E13" s="249"/>
-      <c r="F13" s="249"/>
-      <c r="G13" s="252" t="s">
+      <c r="C13" s="242"/>
+      <c r="D13" s="250"/>
+      <c r="E13" s="251"/>
+      <c r="F13" s="251"/>
+      <c r="G13" s="254" t="s">
         <v>16</v>
       </c>
-      <c r="H13" s="252"/>
-      <c r="I13" s="240"/>
-      <c r="J13" s="255" t="b">
+      <c r="H13" s="254"/>
+      <c r="I13" s="242"/>
+      <c r="J13" s="257" t="b">
         <v>0</v>
       </c>
-      <c r="K13" s="256"/>
-      <c r="L13" s="256" t="b">
+      <c r="K13" s="258"/>
+      <c r="L13" s="258" t="b">
         <v>0</v>
       </c>
-      <c r="M13" s="256"/>
-      <c r="N13" s="257"/>
+      <c r="M13" s="258"/>
+      <c r="N13" s="259"/>
       <c r="P13" s="60" t="s">
         <v>17</v>
       </c>
       <c r="Q13" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="R13" s="272"/>
-      <c r="S13" s="273"/>
-      <c r="T13" s="273"/>
-      <c r="U13" s="273"/>
-      <c r="V13" s="274"/>
+      <c r="R13" s="274"/>
+      <c r="S13" s="275"/>
+      <c r="T13" s="275"/>
+      <c r="U13" s="275"/>
+      <c r="V13" s="276"/>
     </row>
     <row r="14" spans="1:22" ht="21.6" customHeight="1">
       <c r="A14" s="58"/>
       <c r="B14" s="64"/>
       <c r="C14" s="64"/>
-      <c r="D14" s="250"/>
-      <c r="E14" s="251"/>
-      <c r="F14" s="251"/>
-      <c r="G14" s="253"/>
-      <c r="H14" s="253"/>
-      <c r="I14" s="254"/>
-      <c r="J14" s="258" t="b">
+      <c r="D14" s="252"/>
+      <c r="E14" s="253"/>
+      <c r="F14" s="253"/>
+      <c r="G14" s="255"/>
+      <c r="H14" s="255"/>
+      <c r="I14" s="256"/>
+      <c r="J14" s="260" t="b">
         <v>0</v>
       </c>
-      <c r="K14" s="259"/>
-      <c r="L14" s="259" t="b">
+      <c r="K14" s="261"/>
+      <c r="L14" s="261" t="b">
         <v>0</v>
       </c>
-      <c r="M14" s="259"/>
-      <c r="N14" s="260"/>
+      <c r="M14" s="261"/>
+      <c r="N14" s="262"/>
       <c r="P14" s="60"/>
       <c r="Q14" s="2"/>
       <c r="S14"/>
@@ -11216,21 +11222,21 @@
         <v>19</v>
       </c>
       <c r="C15" s="66"/>
-      <c r="D15" s="241"/>
-      <c r="E15" s="241"/>
-      <c r="F15" s="242"/>
-      <c r="G15" s="243" t="s">
+      <c r="D15" s="243"/>
+      <c r="E15" s="243"/>
+      <c r="F15" s="244"/>
+      <c r="G15" s="245" t="s">
         <v>20</v>
       </c>
-      <c r="H15" s="244"/>
-      <c r="I15" s="244"/>
-      <c r="J15" s="245" t="s">
+      <c r="H15" s="246"/>
+      <c r="I15" s="246"/>
+      <c r="J15" s="247" t="s">
         <v>21</v>
       </c>
-      <c r="K15" s="246"/>
-      <c r="L15" s="246"/>
-      <c r="M15" s="246"/>
-      <c r="N15" s="247"/>
+      <c r="K15" s="248"/>
+      <c r="L15" s="248"/>
+      <c r="M15" s="248"/>
+      <c r="N15" s="249"/>
       <c r="P15" s="60" t="s">
         <v>22</v>
       </c>
@@ -11252,22 +11258,22 @@
       <c r="D16" s="1" t="b">
         <v>0</v>
       </c>
-      <c r="E16" s="261" t="b">
+      <c r="E16" s="263" t="b">
         <v>0</v>
       </c>
-      <c r="F16" s="262"/>
-      <c r="G16" s="263" t="s">
+      <c r="F16" s="264"/>
+      <c r="G16" s="265" t="s">
         <v>25</v>
       </c>
-      <c r="H16" s="264"/>
-      <c r="I16" s="265"/>
-      <c r="J16" s="236">
+      <c r="H16" s="266"/>
+      <c r="I16" s="267"/>
+      <c r="J16" s="238">
         <v>1</v>
       </c>
-      <c r="K16" s="237"/>
-      <c r="L16" s="237"/>
-      <c r="M16" s="237"/>
-      <c r="N16" s="238"/>
+      <c r="K16" s="239"/>
+      <c r="L16" s="239"/>
+      <c r="M16" s="239"/>
+      <c r="N16" s="240"/>
       <c r="O16" s="69"/>
       <c r="P16" s="60" t="s">
         <v>26</v>
@@ -11277,60 +11283,60 @@
       </c>
     </row>
     <row r="17" spans="1:23" ht="27" customHeight="1">
-      <c r="A17" s="198">
+      <c r="A17" s="200">
         <v>6</v>
       </c>
-      <c r="B17" s="304" t="s">
+      <c r="B17" s="306" t="s">
         <v>28</v>
       </c>
-      <c r="C17" s="305"/>
+      <c r="C17" s="307"/>
       <c r="D17" s="28" t="b">
         <v>0</v>
       </c>
-      <c r="E17" s="308" t="b">
+      <c r="E17" s="310" t="b">
         <v>0</v>
       </c>
-      <c r="F17" s="309"/>
+      <c r="F17" s="311"/>
       <c r="G17" s="70" t="s">
         <v>29</v>
       </c>
       <c r="H17" s="71"/>
-      <c r="I17" s="197"/>
-      <c r="J17" s="197"/>
-      <c r="K17" s="197"/>
-      <c r="L17" s="197"/>
-      <c r="M17" s="214"/>
-      <c r="N17" s="214"/>
+      <c r="I17" s="199"/>
+      <c r="J17" s="199"/>
+      <c r="K17" s="199"/>
+      <c r="L17" s="199"/>
+      <c r="M17" s="216"/>
+      <c r="N17" s="216"/>
       <c r="Q17" s="2" t="s">
         <v>30</v>
       </c>
       <c r="R17" s="72"/>
     </row>
     <row r="18" spans="1:23" ht="27" customHeight="1">
-      <c r="A18" s="199"/>
-      <c r="B18" s="306"/>
-      <c r="C18" s="307"/>
+      <c r="A18" s="201"/>
+      <c r="B18" s="308"/>
+      <c r="C18" s="309"/>
       <c r="D18" s="29" t="b">
         <v>0</v>
       </c>
-      <c r="E18" s="223" t="b">
+      <c r="E18" s="225" t="b">
         <v>0</v>
       </c>
-      <c r="F18" s="224"/>
+      <c r="F18" s="226"/>
       <c r="G18" s="74"/>
       <c r="H18" s="75"/>
-      <c r="I18" s="218" t="s">
+      <c r="I18" s="220" t="s">
         <v>31</v>
       </c>
-      <c r="J18" s="218"/>
-      <c r="K18" s="218" t="s">
+      <c r="J18" s="220"/>
+      <c r="K18" s="220" t="s">
         <v>337</v>
       </c>
-      <c r="L18" s="218"/>
-      <c r="M18" s="218" t="s">
+      <c r="L18" s="220"/>
+      <c r="M18" s="220" t="s">
         <v>32</v>
       </c>
-      <c r="N18" s="218"/>
+      <c r="N18" s="220"/>
       <c r="Q18" s="2" t="s">
         <v>33</v>
       </c>
@@ -11339,19 +11345,19 @@
       <c r="A19" s="56"/>
       <c r="B19" s="76"/>
       <c r="C19" s="73"/>
-      <c r="D19" s="222" t="b">
+      <c r="D19" s="224" t="b">
         <v>0</v>
       </c>
-      <c r="E19" s="223"/>
-      <c r="F19" s="224"/>
+      <c r="E19" s="225"/>
+      <c r="F19" s="226"/>
       <c r="G19" s="74"/>
       <c r="H19" s="75"/>
-      <c r="I19" s="197"/>
-      <c r="J19" s="214"/>
-      <c r="K19" s="214"/>
-      <c r="L19" s="197"/>
-      <c r="M19" s="214"/>
-      <c r="N19" s="214"/>
+      <c r="I19" s="199"/>
+      <c r="J19" s="216"/>
+      <c r="K19" s="216"/>
+      <c r="L19" s="199"/>
+      <c r="M19" s="216"/>
+      <c r="N19" s="216"/>
       <c r="Q19" s="2" t="s">
         <v>34</v>
       </c>
@@ -11360,67 +11366,67 @@
       <c r="A20" s="77"/>
       <c r="B20" s="78"/>
       <c r="C20" s="79"/>
-      <c r="D20" s="219"/>
-      <c r="E20" s="220"/>
-      <c r="F20" s="221"/>
+      <c r="D20" s="221"/>
+      <c r="E20" s="222"/>
+      <c r="F20" s="223"/>
       <c r="G20" s="58"/>
       <c r="H20" s="59"/>
-      <c r="I20" s="215" t="s">
+      <c r="I20" s="217" t="s">
         <v>35</v>
       </c>
-      <c r="J20" s="216"/>
-      <c r="K20" s="216"/>
-      <c r="L20" s="217" t="s">
+      <c r="J20" s="218"/>
+      <c r="K20" s="218"/>
+      <c r="L20" s="219" t="s">
         <v>36</v>
       </c>
-      <c r="M20" s="303"/>
-      <c r="N20" s="303"/>
+      <c r="M20" s="305"/>
+      <c r="N20" s="305"/>
       <c r="Q20" s="2" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="21" spans="1:23" ht="30.75" customHeight="1">
-      <c r="A21" s="199">
+      <c r="A21" s="201">
         <v>7</v>
       </c>
-      <c r="B21" s="201" t="s">
+      <c r="B21" s="203" t="s">
         <v>38</v>
       </c>
-      <c r="C21" s="202"/>
-      <c r="D21" s="208"/>
-      <c r="E21" s="208"/>
-      <c r="F21" s="208"/>
+      <c r="C21" s="204"/>
+      <c r="D21" s="210"/>
+      <c r="E21" s="210"/>
+      <c r="F21" s="210"/>
       <c r="G21" s="58"/>
       <c r="H21" s="59"/>
-      <c r="I21" s="197"/>
-      <c r="J21" s="214"/>
-      <c r="K21" s="214"/>
-      <c r="L21" s="197"/>
-      <c r="M21" s="214"/>
-      <c r="N21" s="214"/>
+      <c r="I21" s="199"/>
+      <c r="J21" s="216"/>
+      <c r="K21" s="216"/>
+      <c r="L21" s="199"/>
+      <c r="M21" s="216"/>
+      <c r="N21" s="216"/>
       <c r="Q21" s="2" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="22" spans="1:23" ht="26.25" customHeight="1">
-      <c r="A22" s="200"/>
-      <c r="B22" s="203"/>
-      <c r="C22" s="204"/>
-      <c r="D22" s="207"/>
-      <c r="E22" s="207"/>
-      <c r="F22" s="207"/>
+      <c r="A22" s="202"/>
+      <c r="B22" s="205"/>
+      <c r="C22" s="206"/>
+      <c r="D22" s="209"/>
+      <c r="E22" s="209"/>
+      <c r="F22" s="209"/>
       <c r="G22" s="58"/>
       <c r="H22" s="59"/>
-      <c r="I22" s="215" t="s">
+      <c r="I22" s="217" t="s">
         <v>40</v>
       </c>
-      <c r="J22" s="215"/>
-      <c r="K22" s="215"/>
-      <c r="L22" s="217" t="s">
+      <c r="J22" s="217"/>
+      <c r="K22" s="217"/>
+      <c r="L22" s="219" t="s">
         <v>41</v>
       </c>
-      <c r="M22" s="217"/>
-      <c r="N22" s="217"/>
+      <c r="M22" s="219"/>
+      <c r="N22" s="219"/>
       <c r="Q22" s="2" t="s">
         <v>42</v>
       </c>
@@ -11429,166 +11435,166 @@
       <c r="A23" s="56">
         <v>8</v>
       </c>
-      <c r="B23" s="209" t="s">
+      <c r="B23" s="211" t="s">
         <v>43</v>
       </c>
-      <c r="C23" s="210"/>
-      <c r="D23" s="211"/>
-      <c r="E23" s="211"/>
-      <c r="F23" s="211"/>
-      <c r="G23" s="212" t="s">
+      <c r="C23" s="212"/>
+      <c r="D23" s="213"/>
+      <c r="E23" s="213"/>
+      <c r="F23" s="213"/>
+      <c r="G23" s="214" t="s">
         <v>44</v>
       </c>
-      <c r="H23" s="213"/>
-      <c r="I23" s="214"/>
-      <c r="J23" s="214"/>
-      <c r="K23" s="214"/>
-      <c r="L23" s="214"/>
-      <c r="M23" s="214"/>
-      <c r="N23" s="214"/>
+      <c r="H23" s="215"/>
+      <c r="I23" s="216"/>
+      <c r="J23" s="216"/>
+      <c r="K23" s="216"/>
+      <c r="L23" s="216"/>
+      <c r="M23" s="216"/>
+      <c r="N23" s="216"/>
       <c r="Q23" s="2" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="24" spans="1:23" ht="30.75" customHeight="1">
-      <c r="A24" s="198">
+      <c r="A24" s="200">
         <v>9</v>
       </c>
-      <c r="B24" s="201" t="s">
+      <c r="B24" s="203" t="s">
         <v>46</v>
       </c>
-      <c r="C24" s="202"/>
-      <c r="D24" s="206"/>
-      <c r="E24" s="206"/>
-      <c r="F24" s="206"/>
+      <c r="C24" s="204"/>
+      <c r="D24" s="208"/>
+      <c r="E24" s="208"/>
+      <c r="F24" s="208"/>
       <c r="G24" s="82" t="s">
         <v>47</v>
       </c>
       <c r="H24" s="80"/>
-      <c r="I24" s="197"/>
-      <c r="J24" s="197"/>
-      <c r="K24" s="197"/>
-      <c r="L24" s="197"/>
-      <c r="M24" s="214"/>
-      <c r="N24" s="214"/>
+      <c r="I24" s="199"/>
+      <c r="J24" s="199"/>
+      <c r="K24" s="199"/>
+      <c r="L24" s="199"/>
+      <c r="M24" s="216"/>
+      <c r="N24" s="216"/>
       <c r="Q24" s="2" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="25" spans="1:23" ht="29.25" customHeight="1">
-      <c r="A25" s="200"/>
-      <c r="B25" s="203"/>
-      <c r="C25" s="204"/>
-      <c r="D25" s="207"/>
-      <c r="E25" s="207"/>
-      <c r="F25" s="207"/>
+      <c r="A25" s="202"/>
+      <c r="B25" s="205"/>
+      <c r="C25" s="206"/>
+      <c r="D25" s="209"/>
+      <c r="E25" s="209"/>
+      <c r="F25" s="209"/>
       <c r="G25" s="58"/>
       <c r="H25" s="59"/>
-      <c r="I25" s="218" t="s">
+      <c r="I25" s="220" t="s">
         <v>31</v>
       </c>
-      <c r="J25" s="218"/>
-      <c r="K25" s="218" t="s">
+      <c r="J25" s="220"/>
+      <c r="K25" s="220" t="s">
         <v>337</v>
       </c>
-      <c r="L25" s="218"/>
-      <c r="M25" s="218" t="s">
+      <c r="L25" s="220"/>
+      <c r="M25" s="220" t="s">
         <v>32</v>
       </c>
-      <c r="N25" s="218"/>
+      <c r="N25" s="220"/>
       <c r="Q25" s="2" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="26" spans="1:23" ht="29.25" customHeight="1">
-      <c r="A26" s="198">
+      <c r="A26" s="200">
         <v>10</v>
       </c>
-      <c r="B26" s="201" t="s">
+      <c r="B26" s="203" t="s">
         <v>335</v>
       </c>
-      <c r="C26" s="202"/>
-      <c r="D26" s="206"/>
-      <c r="E26" s="206"/>
-      <c r="F26" s="206"/>
+      <c r="C26" s="204"/>
+      <c r="D26" s="208"/>
+      <c r="E26" s="208"/>
+      <c r="F26" s="208"/>
       <c r="G26" s="74"/>
       <c r="H26" s="75"/>
-      <c r="I26" s="197"/>
-      <c r="J26" s="214"/>
-      <c r="K26" s="214"/>
-      <c r="L26" s="197"/>
-      <c r="M26" s="214"/>
-      <c r="N26" s="214"/>
+      <c r="I26" s="199"/>
+      <c r="J26" s="216"/>
+      <c r="K26" s="216"/>
+      <c r="L26" s="199"/>
+      <c r="M26" s="216"/>
+      <c r="N26" s="216"/>
       <c r="Q26" s="2" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="27" spans="1:23" ht="35.25" customHeight="1">
-      <c r="A27" s="200"/>
-      <c r="B27" s="203"/>
-      <c r="C27" s="204"/>
-      <c r="D27" s="207"/>
-      <c r="E27" s="207"/>
-      <c r="F27" s="207"/>
+      <c r="A27" s="202"/>
+      <c r="B27" s="205"/>
+      <c r="C27" s="206"/>
+      <c r="D27" s="209"/>
+      <c r="E27" s="209"/>
+      <c r="F27" s="209"/>
       <c r="G27" s="74"/>
       <c r="H27" s="75"/>
-      <c r="I27" s="215" t="s">
+      <c r="I27" s="217" t="s">
         <v>35</v>
       </c>
-      <c r="J27" s="216"/>
-      <c r="K27" s="216"/>
-      <c r="L27" s="217" t="s">
+      <c r="J27" s="218"/>
+      <c r="K27" s="218"/>
+      <c r="L27" s="219" t="s">
         <v>36</v>
       </c>
-      <c r="M27" s="216"/>
-      <c r="N27" s="216"/>
+      <c r="M27" s="218"/>
+      <c r="N27" s="218"/>
       <c r="Q27" s="2" t="s">
         <v>51</v>
       </c>
       <c r="S27" s="83"/>
     </row>
     <row r="28" spans="1:23" ht="33" customHeight="1">
-      <c r="A28" s="198">
+      <c r="A28" s="200">
         <v>11</v>
       </c>
-      <c r="B28" s="201" t="s">
+      <c r="B28" s="203" t="s">
         <v>52</v>
       </c>
-      <c r="C28" s="202"/>
-      <c r="D28" s="205"/>
-      <c r="E28" s="206"/>
-      <c r="F28" s="206"/>
+      <c r="C28" s="204"/>
+      <c r="D28" s="207"/>
+      <c r="E28" s="208"/>
+      <c r="F28" s="208"/>
       <c r="G28" s="74"/>
       <c r="H28" s="84"/>
-      <c r="I28" s="197"/>
-      <c r="J28" s="214"/>
-      <c r="K28" s="214"/>
-      <c r="L28" s="197"/>
-      <c r="M28" s="214"/>
-      <c r="N28" s="214"/>
+      <c r="I28" s="199"/>
+      <c r="J28" s="216"/>
+      <c r="K28" s="216"/>
+      <c r="L28" s="199"/>
+      <c r="M28" s="216"/>
+      <c r="N28" s="216"/>
       <c r="Q28" s="2" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="29" spans="1:23" ht="32.25" customHeight="1">
-      <c r="A29" s="200"/>
-      <c r="B29" s="203"/>
-      <c r="C29" s="204"/>
-      <c r="D29" s="207"/>
-      <c r="E29" s="207"/>
-      <c r="F29" s="207"/>
+      <c r="A29" s="202"/>
+      <c r="B29" s="205"/>
+      <c r="C29" s="206"/>
+      <c r="D29" s="209"/>
+      <c r="E29" s="209"/>
+      <c r="F29" s="209"/>
       <c r="G29" s="74"/>
       <c r="H29" s="84"/>
-      <c r="I29" s="215" t="s">
+      <c r="I29" s="217" t="s">
         <v>40</v>
       </c>
-      <c r="J29" s="215"/>
-      <c r="K29" s="215"/>
-      <c r="L29" s="215" t="s">
+      <c r="J29" s="217"/>
+      <c r="K29" s="217"/>
+      <c r="L29" s="217" t="s">
         <v>41</v>
       </c>
-      <c r="M29" s="215"/>
-      <c r="N29" s="215"/>
+      <c r="M29" s="217"/>
+      <c r="N29" s="217"/>
       <c r="Q29" s="2" t="s">
         <v>54</v>
       </c>
@@ -11602,19 +11608,19 @@
         <v>55</v>
       </c>
       <c r="C30" s="68"/>
-      <c r="D30" s="205"/>
-      <c r="E30" s="206"/>
-      <c r="F30" s="206"/>
-      <c r="G30" s="212" t="s">
+      <c r="D30" s="207"/>
+      <c r="E30" s="208"/>
+      <c r="F30" s="208"/>
+      <c r="G30" s="214" t="s">
         <v>44</v>
       </c>
-      <c r="H30" s="213"/>
-      <c r="I30" s="214"/>
-      <c r="J30" s="214"/>
-      <c r="K30" s="214"/>
-      <c r="L30" s="214"/>
-      <c r="M30" s="214"/>
-      <c r="N30" s="214"/>
+      <c r="H30" s="215"/>
+      <c r="I30" s="216"/>
+      <c r="J30" s="216"/>
+      <c r="K30" s="216"/>
+      <c r="L30" s="216"/>
+      <c r="M30" s="216"/>
+      <c r="N30" s="216"/>
       <c r="Q30" s="2" t="s">
         <v>56</v>
       </c>
@@ -11631,42 +11637,42 @@
         <v>334</v>
       </c>
       <c r="C31" s="68"/>
-      <c r="D31" s="211"/>
-      <c r="E31" s="211"/>
-      <c r="F31" s="211"/>
+      <c r="D31" s="213"/>
+      <c r="E31" s="213"/>
+      <c r="F31" s="213"/>
       <c r="G31" s="85" t="s">
         <v>57</v>
       </c>
       <c r="H31" s="81"/>
-      <c r="I31" s="197"/>
-      <c r="J31" s="197"/>
-      <c r="K31" s="197"/>
-      <c r="L31" s="197"/>
-      <c r="M31" s="197"/>
-      <c r="N31" s="197"/>
+      <c r="I31" s="199"/>
+      <c r="J31" s="199"/>
+      <c r="K31" s="199"/>
+      <c r="L31" s="199"/>
+      <c r="M31" s="199"/>
+      <c r="N31" s="199"/>
       <c r="Q31" s="2" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="32" spans="1:23" ht="39.75" customHeight="1">
-      <c r="A32" s="225" t="s">
+      <c r="A32" s="227" t="s">
         <v>59</v>
       </c>
-      <c r="B32" s="210"/>
-      <c r="C32" s="226"/>
-      <c r="D32" s="211"/>
-      <c r="E32" s="211"/>
-      <c r="F32" s="211"/>
+      <c r="B32" s="212"/>
+      <c r="C32" s="228"/>
+      <c r="D32" s="213"/>
+      <c r="E32" s="213"/>
+      <c r="F32" s="213"/>
       <c r="G32" s="86" t="s">
         <v>60</v>
       </c>
       <c r="H32" s="87"/>
-      <c r="I32" s="197"/>
-      <c r="J32" s="197"/>
-      <c r="K32" s="197"/>
-      <c r="L32" s="197"/>
-      <c r="M32" s="197"/>
-      <c r="N32" s="197"/>
+      <c r="I32" s="199"/>
+      <c r="J32" s="199"/>
+      <c r="K32" s="199"/>
+      <c r="L32" s="199"/>
+      <c r="M32" s="199"/>
+      <c r="N32" s="199"/>
       <c r="Q32" s="2" t="s">
         <v>61</v>
       </c>
@@ -11675,74 +11681,92 @@
       <c r="A33" s="65">
         <v>15</v>
       </c>
-      <c r="B33" s="301" t="s">
+      <c r="B33" s="303" t="s">
         <v>333</v>
       </c>
-      <c r="C33" s="302"/>
-      <c r="D33" s="298"/>
-      <c r="E33" s="299"/>
-      <c r="F33" s="300"/>
+      <c r="C33" s="304"/>
+      <c r="D33" s="300"/>
+      <c r="E33" s="301"/>
+      <c r="F33" s="302"/>
       <c r="G33" s="88" t="s">
         <v>62</v>
       </c>
       <c r="H33" s="81"/>
-      <c r="I33" s="196"/>
-      <c r="J33" s="197"/>
-      <c r="K33" s="197"/>
-      <c r="L33" s="197"/>
-      <c r="M33" s="197"/>
-      <c r="N33" s="197"/>
+      <c r="I33" s="198"/>
+      <c r="J33" s="199"/>
+      <c r="K33" s="199"/>
+      <c r="L33" s="199"/>
+      <c r="M33" s="199"/>
+      <c r="N33" s="199"/>
       <c r="Q33" s="2" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="34" spans="1:17" ht="16.5" customHeight="1">
-      <c r="A34" s="295" t="s">
+      <c r="A34" s="297" t="s">
         <v>338</v>
       </c>
-      <c r="B34" s="296"/>
-      <c r="C34" s="296"/>
-      <c r="D34" s="296"/>
-      <c r="E34" s="296"/>
-      <c r="F34" s="296"/>
-      <c r="G34" s="296"/>
-      <c r="H34" s="296"/>
-      <c r="I34" s="296"/>
-      <c r="J34" s="296"/>
-      <c r="K34" s="296"/>
-      <c r="L34" s="296"/>
-      <c r="M34" s="296"/>
-      <c r="N34" s="297"/>
+      <c r="B34" s="298"/>
+      <c r="C34" s="298"/>
+      <c r="D34" s="298"/>
+      <c r="E34" s="298"/>
+      <c r="F34" s="298"/>
+      <c r="G34" s="298"/>
+      <c r="H34" s="298"/>
+      <c r="I34" s="298"/>
+      <c r="J34" s="298"/>
+      <c r="K34" s="298"/>
+      <c r="L34" s="298"/>
+      <c r="M34" s="298"/>
+      <c r="N34" s="299"/>
       <c r="Q34" s="2" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="35" spans="1:17" ht="21" customHeight="1">
-      <c r="A35" s="194" t="s">
+      <c r="A35" s="195" t="s">
         <v>339</v>
       </c>
-      <c r="B35" s="194"/>
-      <c r="C35" s="194"/>
-      <c r="D35" s="195" t="s">
+      <c r="B35" s="195"/>
+      <c r="C35" s="195"/>
+      <c r="D35" s="196" t="s">
         <v>341</v>
       </c>
-      <c r="E35" s="195"/>
-      <c r="F35" s="195"/>
-      <c r="G35" s="293" t="s">
+      <c r="E35" s="196"/>
+      <c r="F35" s="196"/>
+      <c r="G35" s="295" t="s">
         <v>340</v>
       </c>
-      <c r="H35" s="294"/>
-      <c r="I35" s="195"/>
-      <c r="J35" s="195"/>
-      <c r="K35" s="195"/>
-      <c r="L35" s="195"/>
-      <c r="M35" s="195"/>
-      <c r="N35" s="195"/>
+      <c r="H35" s="296"/>
+      <c r="I35" s="196"/>
+      <c r="J35" s="196"/>
+      <c r="K35" s="196"/>
+      <c r="L35" s="196"/>
+      <c r="M35" s="196"/>
+      <c r="N35" s="196"/>
       <c r="Q35" s="2" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="36" spans="1:17" ht="21" customHeight="1">
+      <c r="A36" s="195" t="s">
+        <v>345</v>
+      </c>
+      <c r="B36" s="195"/>
+      <c r="C36" s="195"/>
+      <c r="D36" s="196"/>
+      <c r="E36" s="196"/>
+      <c r="F36" s="196"/>
+      <c r="G36" s="197" t="s">
+        <v>340</v>
+      </c>
+      <c r="H36" s="197"/>
+      <c r="I36" s="196"/>
+      <c r="J36" s="196"/>
+      <c r="K36" s="196"/>
+      <c r="L36" s="196"/>
+      <c r="M36" s="196"/>
+      <c r="N36" s="196"/>
       <c r="Q36" s="2" t="s">
         <v>66</v>
       </c>
@@ -15581,9 +15605,8 @@
       <c r="N263" s="90"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="lOkwHRmih2yz9c4Od85lJdM4S+JC/nOIWBrZMwfLY9jIYtNdzhYReltq/WzEz7SyYO0VK1prR0QZLdnQZl+JLQ==" saltValue="P2KUCClITszlOTOmAzsVjQ==" spinCount="100000" sheet="1" scenarios="1"/>
-  <mergeCells count="92">
-    <mergeCell ref="G35:H35"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="wTQYqcELiERpyYppHCKpbis71N72rgw7m/jdydUgASKTdVWlZ9u7OMxN4ialW1ccOV6Lvwl1lRGM2A0otqRrTQ==" saltValue="Rz0L0KmTaKPsJzgMPqdL6Q==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
+  <mergeCells count="96">
     <mergeCell ref="A34:N34"/>
     <mergeCell ref="D33:F33"/>
     <mergeCell ref="B33:C33"/>
@@ -15631,6 +15654,8 @@
     <mergeCell ref="I18:J18"/>
     <mergeCell ref="K18:L18"/>
     <mergeCell ref="M18:N18"/>
+    <mergeCell ref="D20:F20"/>
+    <mergeCell ref="D19:F19"/>
     <mergeCell ref="A32:C32"/>
     <mergeCell ref="D32:F32"/>
     <mergeCell ref="I32:N32"/>
@@ -15641,7 +15666,6 @@
     <mergeCell ref="D30:F30"/>
     <mergeCell ref="G30:H30"/>
     <mergeCell ref="I30:N30"/>
-    <mergeCell ref="D26:F27"/>
     <mergeCell ref="I19:K19"/>
     <mergeCell ref="I26:K26"/>
     <mergeCell ref="L26:N26"/>
@@ -15650,18 +15674,11 @@
     <mergeCell ref="I25:J25"/>
     <mergeCell ref="K25:L25"/>
     <mergeCell ref="M25:N25"/>
-    <mergeCell ref="D20:F20"/>
-    <mergeCell ref="D19:F19"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="D23:F23"/>
-    <mergeCell ref="G23:H23"/>
     <mergeCell ref="I23:N23"/>
     <mergeCell ref="I24:J24"/>
     <mergeCell ref="K24:L24"/>
     <mergeCell ref="M24:N24"/>
-    <mergeCell ref="A35:C35"/>
-    <mergeCell ref="D35:F35"/>
-    <mergeCell ref="I35:N35"/>
+    <mergeCell ref="D26:F27"/>
     <mergeCell ref="I33:N33"/>
     <mergeCell ref="A17:A18"/>
     <mergeCell ref="A21:A22"/>
@@ -15675,10 +15692,24 @@
     <mergeCell ref="B24:C25"/>
     <mergeCell ref="D24:F25"/>
     <mergeCell ref="B26:C27"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="D23:F23"/>
+    <mergeCell ref="G23:H23"/>
+    <mergeCell ref="A36:C36"/>
+    <mergeCell ref="D36:F36"/>
+    <mergeCell ref="G36:H36"/>
+    <mergeCell ref="I36:N36"/>
+    <mergeCell ref="A35:C35"/>
+    <mergeCell ref="D35:F35"/>
+    <mergeCell ref="I35:N35"/>
+    <mergeCell ref="G35:H35"/>
   </mergeCells>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D35" xr:uid="{5EC3205D-4079-402B-BBE7-9B917DF21EB0}">
       <formula1>"Straight, Gay, Lesbian, Bisexual, Pansexual, Asexual, Queer, Prefer not to say, Other(please specify)"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D36:F36" xr:uid="{D6103553-B106-47D6-8124-9A829A70C850}">
+      <formula1>"Tagalog,Cebuano,Dabawenyo,Maranao, Maguindanao, Tausug,Yakan,Sama-Bajau, Badjao, Subanen, Manobo, T'boli, B'laan, Bagobo, Mandaya, Mansaka, Higaonon, Bukidnon, Surigaonon, Kamayo, Chavacano, Tagalog, Ilocano, Ilonggo, Waray, Bicolano, Kapampangan, Other"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
@@ -16186,218 +16217,218 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="3" customHeight="1" thickBot="1">
-      <c r="A1" s="468"/>
-      <c r="B1" s="469"/>
-      <c r="C1" s="469"/>
-      <c r="D1" s="469"/>
-      <c r="E1" s="469"/>
-      <c r="F1" s="469"/>
-      <c r="G1" s="469"/>
-      <c r="H1" s="469"/>
-      <c r="I1" s="469"/>
-      <c r="J1" s="469"/>
+      <c r="A1" s="467"/>
+      <c r="B1" s="468"/>
+      <c r="C1" s="468"/>
+      <c r="D1" s="468"/>
+      <c r="E1" s="468"/>
+      <c r="F1" s="468"/>
+      <c r="G1" s="468"/>
+      <c r="H1" s="468"/>
+      <c r="I1" s="468"/>
+      <c r="J1" s="468"/>
     </row>
     <row r="2" spans="1:15" ht="13.5" customHeight="1">
-      <c r="A2" s="470">
+      <c r="A2" s="469">
         <v>34</v>
       </c>
-      <c r="B2" s="471"/>
-      <c r="C2" s="472" t="s">
+      <c r="B2" s="470"/>
+      <c r="C2" s="471" t="s">
         <v>291</v>
       </c>
-      <c r="D2" s="472"/>
-      <c r="E2" s="472"/>
-      <c r="F2" s="473"/>
-      <c r="G2" s="422"/>
-      <c r="H2" s="423"/>
-      <c r="I2" s="423"/>
-      <c r="J2" s="423"/>
-      <c r="K2" s="423"/>
-      <c r="L2" s="423"/>
-      <c r="M2" s="423"/>
-      <c r="N2" s="423"/>
-      <c r="O2" s="424"/>
+      <c r="D2" s="471"/>
+      <c r="E2" s="471"/>
+      <c r="F2" s="472"/>
+      <c r="G2" s="475"/>
+      <c r="H2" s="476"/>
+      <c r="I2" s="476"/>
+      <c r="J2" s="476"/>
+      <c r="K2" s="476"/>
+      <c r="L2" s="476"/>
+      <c r="M2" s="476"/>
+      <c r="N2" s="476"/>
+      <c r="O2" s="477"/>
     </row>
     <row r="3" spans="1:15" ht="12.75" customHeight="1">
       <c r="A3" s="170"/>
       <c r="B3" s="171"/>
-      <c r="C3" s="474" t="s">
+      <c r="C3" s="473" t="s">
         <v>292</v>
       </c>
-      <c r="D3" s="474"/>
-      <c r="E3" s="474"/>
-      <c r="F3" s="475"/>
-      <c r="G3" s="422"/>
-      <c r="H3" s="423"/>
-      <c r="I3" s="423"/>
-      <c r="J3" s="423"/>
-      <c r="K3" s="423"/>
-      <c r="L3" s="423"/>
-      <c r="M3" s="423"/>
-      <c r="N3" s="423"/>
-      <c r="O3" s="424"/>
+      <c r="D3" s="473"/>
+      <c r="E3" s="473"/>
+      <c r="F3" s="474"/>
+      <c r="G3" s="475"/>
+      <c r="H3" s="476"/>
+      <c r="I3" s="476"/>
+      <c r="J3" s="476"/>
+      <c r="K3" s="476"/>
+      <c r="L3" s="476"/>
+      <c r="M3" s="476"/>
+      <c r="N3" s="476"/>
+      <c r="O3" s="477"/>
     </row>
     <row r="4" spans="1:15">
       <c r="A4" s="170"/>
       <c r="B4" s="171"/>
-      <c r="C4" s="474" t="s">
+      <c r="C4" s="473" t="s">
         <v>293</v>
       </c>
-      <c r="D4" s="474"/>
-      <c r="E4" s="474"/>
-      <c r="F4" s="475"/>
-      <c r="G4" s="422"/>
-      <c r="H4" s="423"/>
-      <c r="I4" s="423"/>
-      <c r="J4" s="423"/>
-      <c r="K4" s="423"/>
-      <c r="L4" s="423"/>
-      <c r="M4" s="423"/>
-      <c r="N4" s="423"/>
-      <c r="O4" s="424"/>
+      <c r="D4" s="473"/>
+      <c r="E4" s="473"/>
+      <c r="F4" s="474"/>
+      <c r="G4" s="475"/>
+      <c r="H4" s="476"/>
+      <c r="I4" s="476"/>
+      <c r="J4" s="476"/>
+      <c r="K4" s="476"/>
+      <c r="L4" s="476"/>
+      <c r="M4" s="476"/>
+      <c r="N4" s="476"/>
+      <c r="O4" s="477"/>
     </row>
     <row r="5" spans="1:15" ht="24.75" customHeight="1">
       <c r="A5" s="170"/>
       <c r="B5" s="171"/>
-      <c r="C5" s="474" t="s">
+      <c r="C5" s="473" t="s">
         <v>294</v>
       </c>
-      <c r="D5" s="474"/>
-      <c r="E5" s="474"/>
-      <c r="F5" s="475"/>
-      <c r="G5" s="432" t="b">
+      <c r="D5" s="473"/>
+      <c r="E5" s="473"/>
+      <c r="F5" s="474"/>
+      <c r="G5" s="431" t="b">
         <v>0</v>
       </c>
-      <c r="H5" s="425"/>
-      <c r="I5" s="425" t="b">
+      <c r="H5" s="424"/>
+      <c r="I5" s="424" t="b">
         <v>0</v>
       </c>
-      <c r="J5" s="425"/>
-      <c r="K5" s="425"/>
-      <c r="L5" s="425"/>
-      <c r="M5" s="425"/>
-      <c r="N5" s="425"/>
-      <c r="O5" s="426"/>
+      <c r="J5" s="424"/>
+      <c r="K5" s="424"/>
+      <c r="L5" s="424"/>
+      <c r="M5" s="424"/>
+      <c r="N5" s="424"/>
+      <c r="O5" s="425"/>
     </row>
     <row r="6" spans="1:15" ht="24" customHeight="1">
       <c r="A6" s="170"/>
       <c r="B6" s="171"/>
-      <c r="C6" s="474" t="s">
+      <c r="C6" s="473" t="s">
         <v>295</v>
       </c>
-      <c r="D6" s="474"/>
-      <c r="E6" s="474"/>
-      <c r="F6" s="475"/>
-      <c r="G6" s="432" t="b">
+      <c r="D6" s="473"/>
+      <c r="E6" s="473"/>
+      <c r="F6" s="474"/>
+      <c r="G6" s="431" t="b">
         <v>0</v>
       </c>
-      <c r="H6" s="425"/>
-      <c r="I6" s="425" t="b">
+      <c r="H6" s="424"/>
+      <c r="I6" s="424" t="b">
         <v>0</v>
       </c>
-      <c r="J6" s="425"/>
-      <c r="K6" s="425"/>
-      <c r="L6" s="425"/>
-      <c r="M6" s="425"/>
-      <c r="N6" s="425"/>
-      <c r="O6" s="426"/>
+      <c r="J6" s="424"/>
+      <c r="K6" s="424"/>
+      <c r="L6" s="424"/>
+      <c r="M6" s="424"/>
+      <c r="N6" s="424"/>
+      <c r="O6" s="425"/>
     </row>
     <row r="7" spans="1:15" ht="27" customHeight="1">
       <c r="A7" s="170"/>
       <c r="B7" s="171"/>
-      <c r="C7" s="474"/>
-      <c r="D7" s="474"/>
-      <c r="E7" s="474"/>
-      <c r="F7" s="474"/>
+      <c r="C7" s="473"/>
+      <c r="D7" s="473"/>
+      <c r="E7" s="473"/>
+      <c r="F7" s="473"/>
       <c r="G7" s="167" t="s">
         <v>318</v>
       </c>
       <c r="H7" s="168"/>
-      <c r="I7" s="427"/>
-      <c r="J7" s="427"/>
-      <c r="K7" s="427"/>
-      <c r="L7" s="427"/>
-      <c r="M7" s="427"/>
-      <c r="N7" s="427"/>
-      <c r="O7" s="428"/>
+      <c r="I7" s="426"/>
+      <c r="J7" s="426"/>
+      <c r="K7" s="426"/>
+      <c r="L7" s="426"/>
+      <c r="M7" s="426"/>
+      <c r="N7" s="426"/>
+      <c r="O7" s="427"/>
     </row>
     <row r="8" spans="1:15" ht="31.5" customHeight="1">
       <c r="A8" s="172"/>
       <c r="B8" s="173"/>
-      <c r="C8" s="478"/>
-      <c r="D8" s="478"/>
-      <c r="E8" s="478"/>
-      <c r="F8" s="479"/>
-      <c r="G8" s="429"/>
-      <c r="H8" s="430"/>
-      <c r="I8" s="430"/>
-      <c r="J8" s="430"/>
-      <c r="K8" s="430"/>
-      <c r="L8" s="430"/>
-      <c r="M8" s="430"/>
-      <c r="N8" s="430"/>
-      <c r="O8" s="431"/>
+      <c r="C8" s="480"/>
+      <c r="D8" s="480"/>
+      <c r="E8" s="480"/>
+      <c r="F8" s="481"/>
+      <c r="G8" s="428"/>
+      <c r="H8" s="429"/>
+      <c r="I8" s="429"/>
+      <c r="J8" s="429"/>
+      <c r="K8" s="429"/>
+      <c r="L8" s="429"/>
+      <c r="M8" s="429"/>
+      <c r="N8" s="429"/>
+      <c r="O8" s="430"/>
     </row>
     <row r="9" spans="1:15" ht="20.45" customHeight="1">
-      <c r="A9" s="480">
+      <c r="A9" s="482">
         <v>35</v>
       </c>
-      <c r="B9" s="481"/>
-      <c r="C9" s="439" t="s">
+      <c r="B9" s="483"/>
+      <c r="C9" s="438" t="s">
         <v>296</v>
       </c>
-      <c r="D9" s="439"/>
-      <c r="E9" s="351"/>
-      <c r="F9" s="482"/>
-      <c r="G9" s="416" t="b">
+      <c r="D9" s="438"/>
+      <c r="E9" s="353"/>
+      <c r="F9" s="484"/>
+      <c r="G9" s="418" t="b">
         <v>0</v>
       </c>
-      <c r="H9" s="417"/>
-      <c r="I9" s="400" t="b">
+      <c r="H9" s="419"/>
+      <c r="I9" s="402" t="b">
         <v>0</v>
       </c>
-      <c r="J9" s="400"/>
-      <c r="K9" s="400"/>
-      <c r="L9" s="400"/>
-      <c r="M9" s="400"/>
-      <c r="N9" s="400"/>
-      <c r="O9" s="401"/>
+      <c r="J9" s="402"/>
+      <c r="K9" s="402"/>
+      <c r="L9" s="402"/>
+      <c r="M9" s="402"/>
+      <c r="N9" s="402"/>
+      <c r="O9" s="403"/>
     </row>
     <row r="10" spans="1:15" ht="26.25" customHeight="1">
       <c r="A10" s="174"/>
       <c r="B10" s="175"/>
-      <c r="C10" s="439"/>
-      <c r="D10" s="439"/>
-      <c r="E10" s="351"/>
-      <c r="F10" s="482"/>
-      <c r="G10" s="490" t="s">
+      <c r="C10" s="438"/>
+      <c r="D10" s="438"/>
+      <c r="E10" s="353"/>
+      <c r="F10" s="484"/>
+      <c r="G10" s="492" t="s">
         <v>318</v>
       </c>
-      <c r="H10" s="491"/>
-      <c r="I10" s="412"/>
-      <c r="J10" s="412"/>
-      <c r="K10" s="412"/>
-      <c r="L10" s="412"/>
-      <c r="M10" s="412"/>
-      <c r="N10" s="412"/>
-      <c r="O10" s="413"/>
+      <c r="H10" s="493"/>
+      <c r="I10" s="414"/>
+      <c r="J10" s="414"/>
+      <c r="K10" s="414"/>
+      <c r="L10" s="414"/>
+      <c r="M10" s="414"/>
+      <c r="N10" s="414"/>
+      <c r="O10" s="415"/>
     </row>
     <row r="11" spans="1:15" ht="21.75" customHeight="1">
       <c r="A11" s="174"/>
       <c r="B11" s="175"/>
-      <c r="C11" s="351"/>
-      <c r="D11" s="351"/>
-      <c r="E11" s="351"/>
-      <c r="F11" s="351"/>
-      <c r="G11" s="497"/>
-      <c r="H11" s="498"/>
-      <c r="I11" s="498"/>
-      <c r="J11" s="498"/>
-      <c r="K11" s="498"/>
-      <c r="L11" s="498"/>
-      <c r="M11" s="498"/>
-      <c r="N11" s="498"/>
-      <c r="O11" s="499"/>
+      <c r="C11" s="353"/>
+      <c r="D11" s="353"/>
+      <c r="E11" s="353"/>
+      <c r="F11" s="353"/>
+      <c r="G11" s="499"/>
+      <c r="H11" s="500"/>
+      <c r="I11" s="500"/>
+      <c r="J11" s="500"/>
+      <c r="K11" s="500"/>
+      <c r="L11" s="500"/>
+      <c r="M11" s="500"/>
+      <c r="N11" s="500"/>
+      <c r="O11" s="501"/>
     </row>
     <row r="12" spans="1:15" ht="18.75" customHeight="1">
       <c r="A12" s="176"/>
@@ -16406,282 +16437,282 @@
       <c r="D12" s="178"/>
       <c r="E12" s="179"/>
       <c r="F12" s="180"/>
-      <c r="G12" s="492" t="b">
+      <c r="G12" s="494" t="b">
         <v>0</v>
       </c>
-      <c r="H12" s="493"/>
-      <c r="I12" s="493" t="b">
+      <c r="H12" s="495"/>
+      <c r="I12" s="495" t="b">
         <v>0</v>
       </c>
-      <c r="J12" s="493"/>
-      <c r="K12" s="493"/>
-      <c r="L12" s="493"/>
-      <c r="M12" s="493"/>
-      <c r="N12" s="493"/>
-      <c r="O12" s="494"/>
+      <c r="J12" s="495"/>
+      <c r="K12" s="495"/>
+      <c r="L12" s="495"/>
+      <c r="M12" s="495"/>
+      <c r="N12" s="495"/>
+      <c r="O12" s="496"/>
     </row>
     <row r="13" spans="1:15" ht="21.75" customHeight="1">
       <c r="A13" s="176"/>
       <c r="B13" s="177"/>
-      <c r="C13" s="483" t="s">
+      <c r="C13" s="485" t="s">
         <v>297</v>
       </c>
-      <c r="D13" s="483"/>
-      <c r="E13" s="484"/>
-      <c r="F13" s="485"/>
-      <c r="G13" s="492"/>
-      <c r="H13" s="493"/>
-      <c r="I13" s="493"/>
-      <c r="J13" s="493"/>
-      <c r="K13" s="493"/>
-      <c r="L13" s="493"/>
-      <c r="M13" s="493"/>
-      <c r="N13" s="493"/>
-      <c r="O13" s="494"/>
+      <c r="D13" s="485"/>
+      <c r="E13" s="486"/>
+      <c r="F13" s="487"/>
+      <c r="G13" s="494"/>
+      <c r="H13" s="495"/>
+      <c r="I13" s="495"/>
+      <c r="J13" s="495"/>
+      <c r="K13" s="495"/>
+      <c r="L13" s="495"/>
+      <c r="M13" s="495"/>
+      <c r="N13" s="495"/>
+      <c r="O13" s="496"/>
     </row>
     <row r="14" spans="1:15" ht="23.25" customHeight="1">
       <c r="A14" s="176"/>
       <c r="B14" s="177"/>
-      <c r="C14" s="483"/>
-      <c r="D14" s="483"/>
-      <c r="E14" s="484"/>
-      <c r="F14" s="485"/>
-      <c r="G14" s="445" t="s">
+      <c r="C14" s="485"/>
+      <c r="D14" s="485"/>
+      <c r="E14" s="486"/>
+      <c r="F14" s="487"/>
+      <c r="G14" s="444" t="s">
         <v>321</v>
       </c>
-      <c r="H14" s="446"/>
-      <c r="I14" s="496"/>
-      <c r="J14" s="496"/>
-      <c r="K14" s="496"/>
-      <c r="L14" s="496"/>
-      <c r="M14" s="496"/>
-      <c r="N14" s="496"/>
-      <c r="O14" s="500"/>
+      <c r="H14" s="445"/>
+      <c r="I14" s="498"/>
+      <c r="J14" s="498"/>
+      <c r="K14" s="498"/>
+      <c r="L14" s="498"/>
+      <c r="M14" s="498"/>
+      <c r="N14" s="498"/>
+      <c r="O14" s="502"/>
     </row>
     <row r="15" spans="1:15" ht="21" customHeight="1">
       <c r="A15" s="176"/>
       <c r="B15" s="177"/>
-      <c r="C15" s="483"/>
-      <c r="D15" s="483"/>
-      <c r="E15" s="484"/>
-      <c r="F15" s="485"/>
-      <c r="G15" s="495" t="s">
+      <c r="C15" s="485"/>
+      <c r="D15" s="485"/>
+      <c r="E15" s="486"/>
+      <c r="F15" s="487"/>
+      <c r="G15" s="497" t="s">
         <v>298</v>
       </c>
-      <c r="H15" s="496"/>
-      <c r="I15" s="412"/>
-      <c r="J15" s="412"/>
-      <c r="K15" s="412"/>
-      <c r="L15" s="412"/>
-      <c r="M15" s="412"/>
-      <c r="N15" s="412"/>
-      <c r="O15" s="413"/>
+      <c r="H15" s="498"/>
+      <c r="I15" s="414"/>
+      <c r="J15" s="414"/>
+      <c r="K15" s="414"/>
+      <c r="L15" s="414"/>
+      <c r="M15" s="414"/>
+      <c r="N15" s="414"/>
+      <c r="O15" s="415"/>
     </row>
     <row r="16" spans="1:15" ht="27.75" customHeight="1">
       <c r="A16" s="176"/>
       <c r="B16" s="177"/>
-      <c r="C16" s="483"/>
-      <c r="D16" s="483"/>
-      <c r="E16" s="484"/>
-      <c r="F16" s="485"/>
-      <c r="G16" s="414" t="s">
+      <c r="C16" s="485"/>
+      <c r="D16" s="485"/>
+      <c r="E16" s="486"/>
+      <c r="F16" s="487"/>
+      <c r="G16" s="416" t="s">
         <v>299</v>
       </c>
-      <c r="H16" s="415"/>
-      <c r="I16" s="420"/>
-      <c r="J16" s="420"/>
-      <c r="K16" s="420"/>
-      <c r="L16" s="420"/>
-      <c r="M16" s="420"/>
-      <c r="N16" s="420"/>
-      <c r="O16" s="421"/>
+      <c r="H16" s="417"/>
+      <c r="I16" s="422"/>
+      <c r="J16" s="422"/>
+      <c r="K16" s="422"/>
+      <c r="L16" s="422"/>
+      <c r="M16" s="422"/>
+      <c r="N16" s="422"/>
+      <c r="O16" s="423"/>
     </row>
     <row r="17" spans="1:15" ht="21" customHeight="1">
       <c r="A17" s="181"/>
       <c r="B17" s="182"/>
-      <c r="C17" s="486"/>
-      <c r="D17" s="486"/>
-      <c r="E17" s="486"/>
-      <c r="F17" s="487"/>
-      <c r="G17" s="409" t="s">
+      <c r="C17" s="488"/>
+      <c r="D17" s="488"/>
+      <c r="E17" s="488"/>
+      <c r="F17" s="489"/>
+      <c r="G17" s="411" t="s">
         <v>300</v>
       </c>
-      <c r="H17" s="410"/>
-      <c r="I17" s="410"/>
-      <c r="J17" s="410"/>
-      <c r="K17" s="410"/>
-      <c r="L17" s="410"/>
-      <c r="M17" s="410"/>
-      <c r="N17" s="410"/>
-      <c r="O17" s="411"/>
+      <c r="H17" s="412"/>
+      <c r="I17" s="412"/>
+      <c r="J17" s="412"/>
+      <c r="K17" s="412"/>
+      <c r="L17" s="412"/>
+      <c r="M17" s="412"/>
+      <c r="N17" s="412"/>
+      <c r="O17" s="413"/>
     </row>
     <row r="18" spans="1:15" ht="33" customHeight="1">
-      <c r="A18" s="476">
+      <c r="A18" s="478">
         <v>36</v>
       </c>
-      <c r="B18" s="477"/>
-      <c r="C18" s="488" t="s">
+      <c r="B18" s="479"/>
+      <c r="C18" s="490" t="s">
         <v>301</v>
       </c>
-      <c r="D18" s="488" t="b">
+      <c r="D18" s="490" t="b">
         <v>0</v>
       </c>
-      <c r="E18" s="488"/>
-      <c r="F18" s="489"/>
-      <c r="G18" s="416" t="b">
+      <c r="E18" s="490"/>
+      <c r="F18" s="491"/>
+      <c r="G18" s="418" t="b">
         <v>0</v>
       </c>
-      <c r="H18" s="417"/>
-      <c r="I18" s="400" t="b">
+      <c r="H18" s="419"/>
+      <c r="I18" s="402" t="b">
         <v>0</v>
       </c>
-      <c r="J18" s="400"/>
-      <c r="K18" s="400"/>
-      <c r="L18" s="400"/>
-      <c r="M18" s="400"/>
-      <c r="N18" s="400"/>
-      <c r="O18" s="401"/>
+      <c r="J18" s="402"/>
+      <c r="K18" s="402"/>
+      <c r="L18" s="402"/>
+      <c r="M18" s="402"/>
+      <c r="N18" s="402"/>
+      <c r="O18" s="403"/>
     </row>
     <row r="19" spans="1:15" ht="26.25" customHeight="1">
       <c r="A19" s="174"/>
       <c r="B19" s="175"/>
-      <c r="C19" s="433"/>
-      <c r="D19" s="433"/>
-      <c r="E19" s="433"/>
-      <c r="F19" s="434"/>
-      <c r="G19" s="418" t="s">
+      <c r="C19" s="432"/>
+      <c r="D19" s="432"/>
+      <c r="E19" s="432"/>
+      <c r="F19" s="433"/>
+      <c r="G19" s="420" t="s">
         <v>320</v>
       </c>
-      <c r="H19" s="419"/>
-      <c r="I19" s="412"/>
-      <c r="J19" s="412"/>
-      <c r="K19" s="412"/>
-      <c r="L19" s="412"/>
-      <c r="M19" s="412"/>
-      <c r="N19" s="412"/>
-      <c r="O19" s="413"/>
+      <c r="H19" s="421"/>
+      <c r="I19" s="414"/>
+      <c r="J19" s="414"/>
+      <c r="K19" s="414"/>
+      <c r="L19" s="414"/>
+      <c r="M19" s="414"/>
+      <c r="N19" s="414"/>
+      <c r="O19" s="415"/>
     </row>
     <row r="20" spans="1:15" ht="25.5" customHeight="1">
       <c r="A20" s="185"/>
       <c r="B20" s="186"/>
-      <c r="C20" s="435"/>
-      <c r="D20" s="435"/>
-      <c r="E20" s="435"/>
-      <c r="F20" s="436"/>
-      <c r="G20" s="409"/>
-      <c r="H20" s="410"/>
-      <c r="I20" s="410"/>
-      <c r="J20" s="410"/>
-      <c r="K20" s="410"/>
-      <c r="L20" s="410"/>
-      <c r="M20" s="410"/>
-      <c r="N20" s="410"/>
-      <c r="O20" s="411"/>
+      <c r="C20" s="434"/>
+      <c r="D20" s="434"/>
+      <c r="E20" s="434"/>
+      <c r="F20" s="435"/>
+      <c r="G20" s="411"/>
+      <c r="H20" s="412"/>
+      <c r="I20" s="412"/>
+      <c r="J20" s="412"/>
+      <c r="K20" s="412"/>
+      <c r="L20" s="412"/>
+      <c r="M20" s="412"/>
+      <c r="N20" s="412"/>
+      <c r="O20" s="413"/>
     </row>
     <row r="21" spans="1:15" ht="26.25" customHeight="1">
-      <c r="A21" s="476">
+      <c r="A21" s="478">
         <v>37</v>
       </c>
-      <c r="B21" s="477"/>
-      <c r="C21" s="488" t="s">
+      <c r="B21" s="479"/>
+      <c r="C21" s="490" t="s">
         <v>302</v>
       </c>
-      <c r="D21" s="488"/>
-      <c r="E21" s="488"/>
-      <c r="F21" s="489"/>
-      <c r="G21" s="416" t="b">
+      <c r="D21" s="490"/>
+      <c r="E21" s="490"/>
+      <c r="F21" s="491"/>
+      <c r="G21" s="418" t="b">
         <v>0</v>
       </c>
-      <c r="H21" s="417"/>
-      <c r="I21" s="400" t="b">
+      <c r="H21" s="419"/>
+      <c r="I21" s="402" t="b">
         <v>0</v>
       </c>
-      <c r="J21" s="400"/>
-      <c r="K21" s="400"/>
-      <c r="L21" s="400"/>
-      <c r="M21" s="400"/>
-      <c r="N21" s="400"/>
-      <c r="O21" s="401"/>
+      <c r="J21" s="402"/>
+      <c r="K21" s="402"/>
+      <c r="L21" s="402"/>
+      <c r="M21" s="402"/>
+      <c r="N21" s="402"/>
+      <c r="O21" s="403"/>
     </row>
     <row r="22" spans="1:15" ht="27.75" customHeight="1">
       <c r="A22" s="174"/>
       <c r="B22" s="175"/>
-      <c r="C22" s="433"/>
-      <c r="D22" s="433"/>
-      <c r="E22" s="433"/>
-      <c r="F22" s="434"/>
-      <c r="G22" s="418" t="s">
+      <c r="C22" s="432"/>
+      <c r="D22" s="432"/>
+      <c r="E22" s="432"/>
+      <c r="F22" s="433"/>
+      <c r="G22" s="420" t="s">
         <v>319</v>
       </c>
-      <c r="H22" s="419"/>
-      <c r="I22" s="412"/>
-      <c r="J22" s="412"/>
-      <c r="K22" s="412"/>
-      <c r="L22" s="412"/>
-      <c r="M22" s="412"/>
-      <c r="N22" s="412"/>
-      <c r="O22" s="413"/>
+      <c r="H22" s="421"/>
+      <c r="I22" s="414"/>
+      <c r="J22" s="414"/>
+      <c r="K22" s="414"/>
+      <c r="L22" s="414"/>
+      <c r="M22" s="414"/>
+      <c r="N22" s="414"/>
+      <c r="O22" s="415"/>
     </row>
     <row r="23" spans="1:15" ht="39.75" customHeight="1">
       <c r="A23" s="185"/>
       <c r="B23" s="186"/>
-      <c r="C23" s="435"/>
-      <c r="D23" s="435"/>
-      <c r="E23" s="435"/>
-      <c r="F23" s="436"/>
-      <c r="G23" s="409"/>
-      <c r="H23" s="410"/>
-      <c r="I23" s="410"/>
-      <c r="J23" s="410"/>
-      <c r="K23" s="410"/>
-      <c r="L23" s="410"/>
-      <c r="M23" s="410"/>
-      <c r="N23" s="410"/>
-      <c r="O23" s="411"/>
+      <c r="C23" s="434"/>
+      <c r="D23" s="434"/>
+      <c r="E23" s="434"/>
+      <c r="F23" s="435"/>
+      <c r="G23" s="411"/>
+      <c r="H23" s="412"/>
+      <c r="I23" s="412"/>
+      <c r="J23" s="412"/>
+      <c r="K23" s="412"/>
+      <c r="L23" s="412"/>
+      <c r="M23" s="412"/>
+      <c r="N23" s="412"/>
+      <c r="O23" s="413"/>
     </row>
     <row r="24" spans="1:15" ht="38.25" customHeight="1">
-      <c r="A24" s="476">
+      <c r="A24" s="478">
         <v>38</v>
       </c>
-      <c r="B24" s="477"/>
-      <c r="C24" s="488" t="s">
+      <c r="B24" s="479"/>
+      <c r="C24" s="490" t="s">
         <v>303</v>
       </c>
-      <c r="D24" s="488"/>
-      <c r="E24" s="488"/>
-      <c r="F24" s="489"/>
-      <c r="G24" s="416" t="b">
+      <c r="D24" s="490"/>
+      <c r="E24" s="490"/>
+      <c r="F24" s="491"/>
+      <c r="G24" s="418" t="b">
         <v>0</v>
       </c>
-      <c r="H24" s="417"/>
-      <c r="I24" s="400" t="b">
+      <c r="H24" s="419"/>
+      <c r="I24" s="402" t="b">
         <v>0</v>
       </c>
-      <c r="J24" s="400"/>
-      <c r="K24" s="400"/>
-      <c r="L24" s="400"/>
-      <c r="M24" s="400"/>
-      <c r="N24" s="400"/>
-      <c r="O24" s="401"/>
+      <c r="J24" s="402"/>
+      <c r="K24" s="402"/>
+      <c r="L24" s="402"/>
+      <c r="M24" s="402"/>
+      <c r="N24" s="402"/>
+      <c r="O24" s="403"/>
     </row>
     <row r="25" spans="1:15" ht="28.5" customHeight="1">
       <c r="A25" s="174"/>
       <c r="B25" s="175"/>
-      <c r="C25" s="433"/>
-      <c r="D25" s="433"/>
-      <c r="E25" s="433"/>
-      <c r="F25" s="434"/>
-      <c r="G25" s="445" t="s">
+      <c r="C25" s="432"/>
+      <c r="D25" s="432"/>
+      <c r="E25" s="432"/>
+      <c r="F25" s="433"/>
+      <c r="G25" s="444" t="s">
         <v>304</v>
       </c>
-      <c r="H25" s="446"/>
-      <c r="I25" s="402"/>
-      <c r="J25" s="402"/>
-      <c r="K25" s="402"/>
-      <c r="L25" s="402"/>
-      <c r="M25" s="402"/>
-      <c r="N25" s="402"/>
-      <c r="O25" s="403"/>
+      <c r="H25" s="445"/>
+      <c r="I25" s="404"/>
+      <c r="J25" s="404"/>
+      <c r="K25" s="404"/>
+      <c r="L25" s="404"/>
+      <c r="M25" s="404"/>
+      <c r="N25" s="404"/>
+      <c r="O25" s="405"/>
     </row>
     <row r="26" spans="1:15" ht="23.25" customHeight="1">
       <c r="A26" s="174"/>
@@ -16690,237 +16721,237 @@
       <c r="D26" s="183"/>
       <c r="E26" s="183"/>
       <c r="F26" s="184"/>
-      <c r="G26" s="443" t="b">
+      <c r="G26" s="442" t="b">
         <v>0</v>
       </c>
-      <c r="H26" s="444"/>
-      <c r="I26" s="404" t="b">
+      <c r="H26" s="443"/>
+      <c r="I26" s="406" t="b">
         <v>0</v>
       </c>
-      <c r="J26" s="404"/>
-      <c r="K26" s="404"/>
-      <c r="L26" s="404"/>
-      <c r="M26" s="404"/>
-      <c r="N26" s="404"/>
-      <c r="O26" s="405"/>
+      <c r="J26" s="406"/>
+      <c r="K26" s="406"/>
+      <c r="L26" s="406"/>
+      <c r="M26" s="406"/>
+      <c r="N26" s="406"/>
+      <c r="O26" s="407"/>
     </row>
     <row r="27" spans="1:15" ht="24.75" customHeight="1">
       <c r="A27" s="174"/>
       <c r="B27" s="175"/>
-      <c r="C27" s="433" t="s">
+      <c r="C27" s="432" t="s">
         <v>305</v>
       </c>
-      <c r="D27" s="433"/>
-      <c r="E27" s="433"/>
-      <c r="F27" s="434"/>
-      <c r="G27" s="443"/>
-      <c r="H27" s="444"/>
-      <c r="I27" s="406"/>
-      <c r="J27" s="406"/>
-      <c r="K27" s="406"/>
-      <c r="L27" s="406"/>
-      <c r="M27" s="406"/>
-      <c r="N27" s="406"/>
-      <c r="O27" s="407"/>
+      <c r="D27" s="432"/>
+      <c r="E27" s="432"/>
+      <c r="F27" s="433"/>
+      <c r="G27" s="442"/>
+      <c r="H27" s="443"/>
+      <c r="I27" s="408"/>
+      <c r="J27" s="408"/>
+      <c r="K27" s="408"/>
+      <c r="L27" s="408"/>
+      <c r="M27" s="408"/>
+      <c r="N27" s="408"/>
+      <c r="O27" s="409"/>
     </row>
     <row r="28" spans="1:15" ht="36" customHeight="1">
       <c r="A28" s="174"/>
       <c r="B28" s="175"/>
-      <c r="C28" s="433"/>
-      <c r="D28" s="433"/>
-      <c r="E28" s="433"/>
-      <c r="F28" s="434"/>
-      <c r="G28" s="445" t="s">
+      <c r="C28" s="432"/>
+      <c r="D28" s="432"/>
+      <c r="E28" s="432"/>
+      <c r="F28" s="433"/>
+      <c r="G28" s="444" t="s">
         <v>304</v>
       </c>
-      <c r="H28" s="446"/>
-      <c r="I28" s="402"/>
-      <c r="J28" s="402"/>
-      <c r="K28" s="402"/>
-      <c r="L28" s="402"/>
-      <c r="M28" s="402"/>
-      <c r="N28" s="402"/>
-      <c r="O28" s="403"/>
+      <c r="H28" s="445"/>
+      <c r="I28" s="404"/>
+      <c r="J28" s="404"/>
+      <c r="K28" s="404"/>
+      <c r="L28" s="404"/>
+      <c r="M28" s="404"/>
+      <c r="N28" s="404"/>
+      <c r="O28" s="405"/>
     </row>
     <row r="29" spans="1:15" ht="30.75" customHeight="1">
       <c r="A29" s="185"/>
       <c r="B29" s="186"/>
-      <c r="C29" s="435"/>
-      <c r="D29" s="435"/>
-      <c r="E29" s="435"/>
-      <c r="F29" s="436"/>
-      <c r="G29" s="447"/>
-      <c r="H29" s="448"/>
-      <c r="I29" s="448"/>
-      <c r="J29" s="448"/>
-      <c r="K29" s="448"/>
-      <c r="L29" s="448"/>
-      <c r="M29" s="448"/>
-      <c r="N29" s="448"/>
-      <c r="O29" s="449"/>
+      <c r="C29" s="434"/>
+      <c r="D29" s="434"/>
+      <c r="E29" s="434"/>
+      <c r="F29" s="435"/>
+      <c r="G29" s="446"/>
+      <c r="H29" s="447"/>
+      <c r="I29" s="447"/>
+      <c r="J29" s="447"/>
+      <c r="K29" s="447"/>
+      <c r="L29" s="447"/>
+      <c r="M29" s="447"/>
+      <c r="N29" s="447"/>
+      <c r="O29" s="448"/>
     </row>
     <row r="30" spans="1:15" ht="23.45" customHeight="1">
-      <c r="A30" s="476">
+      <c r="A30" s="478">
         <v>39</v>
       </c>
-      <c r="B30" s="477"/>
-      <c r="C30" s="437" t="s">
+      <c r="B30" s="479"/>
+      <c r="C30" s="436" t="s">
         <v>306</v>
       </c>
-      <c r="D30" s="437"/>
-      <c r="E30" s="437"/>
-      <c r="F30" s="438"/>
-      <c r="G30" s="416" t="b">
+      <c r="D30" s="436"/>
+      <c r="E30" s="436"/>
+      <c r="F30" s="437"/>
+      <c r="G30" s="418" t="b">
         <v>0</v>
       </c>
-      <c r="H30" s="417"/>
-      <c r="I30" s="400" t="b">
+      <c r="H30" s="419"/>
+      <c r="I30" s="402" t="b">
         <v>0</v>
       </c>
-      <c r="J30" s="400"/>
-      <c r="K30" s="400"/>
-      <c r="L30" s="400"/>
-      <c r="M30" s="400"/>
-      <c r="N30" s="400"/>
-      <c r="O30" s="401"/>
+      <c r="J30" s="402"/>
+      <c r="K30" s="402"/>
+      <c r="L30" s="402"/>
+      <c r="M30" s="402"/>
+      <c r="N30" s="402"/>
+      <c r="O30" s="403"/>
     </row>
     <row r="31" spans="1:15" ht="27" customHeight="1">
       <c r="A31" s="174"/>
       <c r="B31" s="175"/>
-      <c r="C31" s="439"/>
-      <c r="D31" s="439"/>
-      <c r="E31" s="439"/>
-      <c r="F31" s="440"/>
-      <c r="G31" s="418" t="s">
+      <c r="C31" s="438"/>
+      <c r="D31" s="438"/>
+      <c r="E31" s="438"/>
+      <c r="F31" s="439"/>
+      <c r="G31" s="420" t="s">
         <v>307</v>
       </c>
-      <c r="H31" s="419"/>
-      <c r="I31" s="450"/>
-      <c r="J31" s="450"/>
-      <c r="K31" s="450"/>
-      <c r="L31" s="450"/>
-      <c r="M31" s="450"/>
-      <c r="N31" s="450"/>
-      <c r="O31" s="451"/>
+      <c r="H31" s="421"/>
+      <c r="I31" s="449"/>
+      <c r="J31" s="449"/>
+      <c r="K31" s="449"/>
+      <c r="L31" s="449"/>
+      <c r="M31" s="449"/>
+      <c r="N31" s="449"/>
+      <c r="O31" s="450"/>
     </row>
     <row r="32" spans="1:15" ht="33.75" customHeight="1">
       <c r="A32" s="185"/>
       <c r="B32" s="186"/>
-      <c r="C32" s="441"/>
-      <c r="D32" s="441"/>
-      <c r="E32" s="441"/>
-      <c r="F32" s="442"/>
-      <c r="G32" s="452"/>
-      <c r="H32" s="453"/>
-      <c r="I32" s="453"/>
-      <c r="J32" s="453"/>
-      <c r="K32" s="453"/>
-      <c r="L32" s="453"/>
-      <c r="M32" s="453"/>
-      <c r="N32" s="453"/>
-      <c r="O32" s="454"/>
+      <c r="C32" s="440"/>
+      <c r="D32" s="440"/>
+      <c r="E32" s="440"/>
+      <c r="F32" s="441"/>
+      <c r="G32" s="451"/>
+      <c r="H32" s="452"/>
+      <c r="I32" s="452"/>
+      <c r="J32" s="452"/>
+      <c r="K32" s="452"/>
+      <c r="L32" s="452"/>
+      <c r="M32" s="452"/>
+      <c r="N32" s="452"/>
+      <c r="O32" s="453"/>
     </row>
     <row r="33" spans="1:15" ht="46.5" customHeight="1">
-      <c r="A33" s="463">
+      <c r="A33" s="462">
         <v>40</v>
       </c>
-      <c r="B33" s="464"/>
-      <c r="C33" s="433" t="s">
+      <c r="B33" s="463"/>
+      <c r="C33" s="432" t="s">
         <v>308</v>
       </c>
-      <c r="D33" s="433"/>
-      <c r="E33" s="433"/>
-      <c r="F33" s="434"/>
-      <c r="G33" s="465"/>
-      <c r="H33" s="466"/>
-      <c r="I33" s="466"/>
-      <c r="J33" s="466"/>
-      <c r="K33" s="466"/>
-      <c r="L33" s="466"/>
-      <c r="M33" s="466"/>
-      <c r="N33" s="466"/>
-      <c r="O33" s="467"/>
+      <c r="D33" s="432"/>
+      <c r="E33" s="432"/>
+      <c r="F33" s="433"/>
+      <c r="G33" s="464"/>
+      <c r="H33" s="465"/>
+      <c r="I33" s="465"/>
+      <c r="J33" s="465"/>
+      <c r="K33" s="465"/>
+      <c r="L33" s="465"/>
+      <c r="M33" s="465"/>
+      <c r="N33" s="465"/>
+      <c r="O33" s="466"/>
     </row>
     <row r="34" spans="1:15" ht="39.75" customHeight="1">
       <c r="A34" s="187" t="s">
         <v>309</v>
       </c>
       <c r="B34" s="188"/>
-      <c r="C34" s="433" t="s">
+      <c r="C34" s="432" t="s">
         <v>310</v>
       </c>
-      <c r="D34" s="433"/>
-      <c r="E34" s="433"/>
-      <c r="F34" s="434"/>
-      <c r="G34" s="432" t="b">
+      <c r="D34" s="432"/>
+      <c r="E34" s="432"/>
+      <c r="F34" s="433"/>
+      <c r="G34" s="431" t="b">
         <v>0</v>
       </c>
-      <c r="H34" s="425"/>
-      <c r="I34" s="425" t="b">
+      <c r="H34" s="424"/>
+      <c r="I34" s="424" t="b">
         <v>0</v>
       </c>
-      <c r="J34" s="425"/>
-      <c r="K34" s="425"/>
-      <c r="L34" s="425"/>
-      <c r="M34" s="425"/>
-      <c r="N34" s="425"/>
-      <c r="O34" s="426"/>
+      <c r="J34" s="424"/>
+      <c r="K34" s="424"/>
+      <c r="L34" s="424"/>
+      <c r="M34" s="424"/>
+      <c r="N34" s="424"/>
+      <c r="O34" s="425"/>
     </row>
     <row r="35" spans="1:15" ht="36.75" customHeight="1">
       <c r="A35" s="189"/>
       <c r="B35" s="188"/>
-      <c r="C35" s="433"/>
-      <c r="D35" s="433"/>
-      <c r="E35" s="433"/>
-      <c r="F35" s="434"/>
-      <c r="G35" s="445" t="s">
+      <c r="C35" s="432"/>
+      <c r="D35" s="432"/>
+      <c r="E35" s="432"/>
+      <c r="F35" s="433"/>
+      <c r="G35" s="444" t="s">
         <v>304</v>
       </c>
-      <c r="H35" s="446"/>
-      <c r="I35" s="450"/>
-      <c r="J35" s="450"/>
-      <c r="K35" s="450"/>
-      <c r="L35" s="450"/>
-      <c r="M35" s="450"/>
-      <c r="N35" s="450"/>
-      <c r="O35" s="451"/>
+      <c r="H35" s="445"/>
+      <c r="I35" s="449"/>
+      <c r="J35" s="449"/>
+      <c r="K35" s="449"/>
+      <c r="L35" s="449"/>
+      <c r="M35" s="449"/>
+      <c r="N35" s="449"/>
+      <c r="O35" s="450"/>
     </row>
     <row r="36" spans="1:15" ht="33" customHeight="1">
       <c r="A36" s="187" t="s">
         <v>311</v>
       </c>
       <c r="B36" s="188"/>
-      <c r="C36" s="434" t="s">
+      <c r="C36" s="433" t="s">
         <v>312</v>
       </c>
-      <c r="D36" s="434"/>
-      <c r="E36" s="434"/>
-      <c r="F36" s="434"/>
-      <c r="G36" s="432" t="b">
+      <c r="D36" s="433"/>
+      <c r="E36" s="433"/>
+      <c r="F36" s="433"/>
+      <c r="G36" s="431" t="b">
         <v>0</v>
       </c>
-      <c r="H36" s="425"/>
-      <c r="I36" s="460" t="b">
+      <c r="H36" s="424"/>
+      <c r="I36" s="459" t="b">
         <v>0</v>
       </c>
-      <c r="J36" s="460"/>
-      <c r="K36" s="460"/>
-      <c r="L36" s="460"/>
-      <c r="M36" s="460"/>
-      <c r="N36" s="460"/>
-      <c r="O36" s="461"/>
+      <c r="J36" s="459"/>
+      <c r="K36" s="459"/>
+      <c r="L36" s="459"/>
+      <c r="M36" s="459"/>
+      <c r="N36" s="459"/>
+      <c r="O36" s="460"/>
     </row>
     <row r="37" spans="1:15" ht="27.75" customHeight="1">
       <c r="A37" s="189"/>
       <c r="B37" s="188"/>
-      <c r="C37" s="434"/>
-      <c r="D37" s="434"/>
-      <c r="E37" s="434"/>
-      <c r="F37" s="434"/>
-      <c r="G37" s="445" t="s">
+      <c r="C37" s="433"/>
+      <c r="D37" s="433"/>
+      <c r="E37" s="433"/>
+      <c r="F37" s="433"/>
+      <c r="G37" s="444" t="s">
         <v>304</v>
       </c>
-      <c r="H37" s="446"/>
+      <c r="H37" s="445"/>
       <c r="I37" s="29" t="b">
         <v>0</v>
       </c>
@@ -16948,16 +16979,16 @@
         <v>313</v>
       </c>
       <c r="B38" s="188"/>
-      <c r="C38" s="433" t="s">
+      <c r="C38" s="432" t="s">
         <v>314</v>
       </c>
-      <c r="D38" s="433"/>
+      <c r="D38" s="432"/>
       <c r="E38" s="190"/>
       <c r="F38" s="191"/>
-      <c r="G38" s="455" t="b">
+      <c r="G38" s="454" t="b">
         <v>0</v>
       </c>
-      <c r="H38" s="456"/>
+      <c r="H38" s="455"/>
       <c r="I38" s="166" t="b">
         <v>0</v>
       </c>
@@ -16969,133 +17000,133 @@
       <c r="O38" s="169"/>
     </row>
     <row r="39" spans="1:15" ht="28.5" customHeight="1">
-      <c r="A39" s="457"/>
-      <c r="B39" s="458"/>
-      <c r="C39" s="458"/>
-      <c r="D39" s="458"/>
-      <c r="E39" s="458"/>
-      <c r="F39" s="459"/>
-      <c r="G39" s="445" t="s">
+      <c r="A39" s="456"/>
+      <c r="B39" s="457"/>
+      <c r="C39" s="457"/>
+      <c r="D39" s="457"/>
+      <c r="E39" s="457"/>
+      <c r="F39" s="458"/>
+      <c r="G39" s="444" t="s">
         <v>304</v>
       </c>
-      <c r="H39" s="446"/>
-      <c r="I39" s="450"/>
-      <c r="J39" s="450"/>
-      <c r="K39" s="450"/>
-      <c r="L39" s="450"/>
-      <c r="M39" s="450"/>
-      <c r="N39" s="450"/>
-      <c r="O39" s="451"/>
+      <c r="H39" s="445"/>
+      <c r="I39" s="449"/>
+      <c r="J39" s="449"/>
+      <c r="K39" s="449"/>
+      <c r="L39" s="449"/>
+      <c r="M39" s="449"/>
+      <c r="N39" s="449"/>
+      <c r="O39" s="450"/>
     </row>
     <row r="40" spans="1:15" ht="37.5" customHeight="1">
-      <c r="A40" s="457"/>
-      <c r="B40" s="458"/>
-      <c r="C40" s="458"/>
-      <c r="D40" s="458"/>
-      <c r="E40" s="458"/>
-      <c r="F40" s="459"/>
-      <c r="G40" s="445"/>
-      <c r="H40" s="446"/>
-      <c r="I40" s="446"/>
-      <c r="J40" s="446"/>
-      <c r="K40" s="446"/>
-      <c r="L40" s="446"/>
-      <c r="M40" s="446"/>
-      <c r="N40" s="446"/>
-      <c r="O40" s="462"/>
+      <c r="A40" s="456"/>
+      <c r="B40" s="457"/>
+      <c r="C40" s="457"/>
+      <c r="D40" s="457"/>
+      <c r="E40" s="457"/>
+      <c r="F40" s="458"/>
+      <c r="G40" s="444"/>
+      <c r="H40" s="445"/>
+      <c r="I40" s="445"/>
+      <c r="J40" s="445"/>
+      <c r="K40" s="445"/>
+      <c r="L40" s="445"/>
+      <c r="M40" s="445"/>
+      <c r="N40" s="445"/>
+      <c r="O40" s="461"/>
     </row>
     <row r="41" spans="1:15" ht="23.25" customHeight="1">
-      <c r="A41" s="397" t="s">
+      <c r="A41" s="399" t="s">
         <v>342</v>
       </c>
-      <c r="B41" s="397"/>
-      <c r="C41" s="397"/>
-      <c r="D41" s="397"/>
-      <c r="E41" s="397"/>
-      <c r="F41" s="397"/>
-      <c r="G41" s="397"/>
-      <c r="H41" s="397"/>
-      <c r="I41" s="397"/>
-      <c r="J41" s="397"/>
-      <c r="K41" s="397"/>
-      <c r="L41" s="397"/>
-      <c r="M41" s="397"/>
-      <c r="N41" s="397"/>
-      <c r="O41" s="397"/>
+      <c r="B41" s="399"/>
+      <c r="C41" s="399"/>
+      <c r="D41" s="399"/>
+      <c r="E41" s="399"/>
+      <c r="F41" s="399"/>
+      <c r="G41" s="399"/>
+      <c r="H41" s="399"/>
+      <c r="I41" s="399"/>
+      <c r="J41" s="399"/>
+      <c r="K41" s="399"/>
+      <c r="L41" s="399"/>
+      <c r="M41" s="399"/>
+      <c r="N41" s="399"/>
+      <c r="O41" s="399"/>
     </row>
     <row r="42" spans="1:15" ht="18" customHeight="1">
-      <c r="A42" s="398" t="s">
+      <c r="A42" s="400" t="s">
         <v>315</v>
       </c>
-      <c r="B42" s="398"/>
-      <c r="C42" s="398"/>
-      <c r="D42" s="398"/>
-      <c r="E42" s="398"/>
-      <c r="F42" s="398"/>
-      <c r="G42" s="398" t="s">
+      <c r="B42" s="400"/>
+      <c r="C42" s="400"/>
+      <c r="D42" s="400"/>
+      <c r="E42" s="400"/>
+      <c r="F42" s="400"/>
+      <c r="G42" s="400" t="s">
         <v>316</v>
       </c>
-      <c r="H42" s="398"/>
-      <c r="I42" s="398"/>
-      <c r="J42" s="398"/>
-      <c r="K42" s="398"/>
-      <c r="L42" s="398"/>
-      <c r="M42" s="408" t="s">
+      <c r="H42" s="400"/>
+      <c r="I42" s="400"/>
+      <c r="J42" s="400"/>
+      <c r="K42" s="400"/>
+      <c r="L42" s="400"/>
+      <c r="M42" s="410" t="s">
         <v>317</v>
       </c>
-      <c r="N42" s="408"/>
-      <c r="O42" s="408"/>
+      <c r="N42" s="410"/>
+      <c r="O42" s="410"/>
     </row>
     <row r="43" spans="1:15" ht="24" customHeight="1">
-      <c r="A43" s="399"/>
-      <c r="B43" s="399"/>
-      <c r="C43" s="399"/>
-      <c r="D43" s="399"/>
-      <c r="E43" s="399"/>
-      <c r="F43" s="399"/>
-      <c r="G43" s="396"/>
-      <c r="H43" s="396"/>
-      <c r="I43" s="396"/>
-      <c r="J43" s="396"/>
-      <c r="K43" s="396"/>
-      <c r="L43" s="396"/>
-      <c r="M43" s="396"/>
-      <c r="N43" s="396"/>
-      <c r="O43" s="396"/>
+      <c r="A43" s="401"/>
+      <c r="B43" s="401"/>
+      <c r="C43" s="401"/>
+      <c r="D43" s="401"/>
+      <c r="E43" s="401"/>
+      <c r="F43" s="401"/>
+      <c r="G43" s="398"/>
+      <c r="H43" s="398"/>
+      <c r="I43" s="398"/>
+      <c r="J43" s="398"/>
+      <c r="K43" s="398"/>
+      <c r="L43" s="398"/>
+      <c r="M43" s="398"/>
+      <c r="N43" s="398"/>
+      <c r="O43" s="398"/>
     </row>
     <row r="44" spans="1:15" ht="24" customHeight="1">
-      <c r="A44" s="399"/>
-      <c r="B44" s="399"/>
-      <c r="C44" s="399"/>
-      <c r="D44" s="399"/>
-      <c r="E44" s="399"/>
-      <c r="F44" s="399"/>
-      <c r="G44" s="396"/>
-      <c r="H44" s="396"/>
-      <c r="I44" s="396"/>
-      <c r="J44" s="396"/>
-      <c r="K44" s="396"/>
-      <c r="L44" s="396"/>
-      <c r="M44" s="396"/>
-      <c r="N44" s="396"/>
-      <c r="O44" s="396"/>
+      <c r="A44" s="401"/>
+      <c r="B44" s="401"/>
+      <c r="C44" s="401"/>
+      <c r="D44" s="401"/>
+      <c r="E44" s="401"/>
+      <c r="F44" s="401"/>
+      <c r="G44" s="398"/>
+      <c r="H44" s="398"/>
+      <c r="I44" s="398"/>
+      <c r="J44" s="398"/>
+      <c r="K44" s="398"/>
+      <c r="L44" s="398"/>
+      <c r="M44" s="398"/>
+      <c r="N44" s="398"/>
+      <c r="O44" s="398"/>
     </row>
     <row r="45" spans="1:15" ht="24" customHeight="1">
-      <c r="A45" s="399"/>
-      <c r="B45" s="399"/>
-      <c r="C45" s="399"/>
-      <c r="D45" s="399"/>
-      <c r="E45" s="399"/>
-      <c r="F45" s="399"/>
-      <c r="G45" s="396"/>
-      <c r="H45" s="396"/>
-      <c r="I45" s="396"/>
-      <c r="J45" s="396"/>
-      <c r="K45" s="396"/>
-      <c r="L45" s="396"/>
-      <c r="M45" s="396"/>
-      <c r="N45" s="396"/>
-      <c r="O45" s="396"/>
+      <c r="A45" s="401"/>
+      <c r="B45" s="401"/>
+      <c r="C45" s="401"/>
+      <c r="D45" s="401"/>
+      <c r="E45" s="401"/>
+      <c r="F45" s="401"/>
+      <c r="G45" s="398"/>
+      <c r="H45" s="398"/>
+      <c r="I45" s="398"/>
+      <c r="J45" s="398"/>
+      <c r="K45" s="398"/>
+      <c r="L45" s="398"/>
+      <c r="M45" s="398"/>
+      <c r="N45" s="398"/>
+      <c r="O45" s="398"/>
     </row>
     <row r="46" spans="1:15" ht="25.5" customHeight="1"/>
     <row r="47" spans="1:15" ht="24.75" customHeight="1"/>
@@ -17152,6 +17183,7 @@
     <mergeCell ref="C2:F2"/>
     <mergeCell ref="C3:F3"/>
     <mergeCell ref="C4:F4"/>
+    <mergeCell ref="G2:O4"/>
     <mergeCell ref="A33:B33"/>
     <mergeCell ref="G35:H35"/>
     <mergeCell ref="G34:H34"/>
@@ -17179,7 +17211,6 @@
     <mergeCell ref="I30:O30"/>
     <mergeCell ref="I31:O31"/>
     <mergeCell ref="G32:O32"/>
-    <mergeCell ref="G2:O4"/>
     <mergeCell ref="I5:O5"/>
     <mergeCell ref="I6:O6"/>
     <mergeCell ref="I7:O7"/>
@@ -17926,223 +17957,223 @@
       <c r="A1" s="92" t="s">
         <v>246</v>
       </c>
-      <c r="B1" s="330" t="s">
+      <c r="B1" s="332" t="s">
         <v>247</v>
       </c>
-      <c r="C1" s="330"/>
-      <c r="D1" s="330"/>
-      <c r="E1" s="330"/>
-      <c r="F1" s="330"/>
-      <c r="G1" s="330"/>
-      <c r="H1" s="330"/>
-      <c r="I1" s="330"/>
-      <c r="J1" s="330"/>
+      <c r="C1" s="332"/>
+      <c r="D1" s="332"/>
+      <c r="E1" s="332"/>
+      <c r="F1" s="332"/>
+      <c r="G1" s="332"/>
+      <c r="H1" s="332"/>
+      <c r="I1" s="332"/>
+      <c r="J1" s="332"/>
     </row>
     <row r="2" spans="1:10" ht="21" customHeight="1">
       <c r="A2" s="93">
         <v>22</v>
       </c>
-      <c r="B2" s="322" t="s">
+      <c r="B2" s="324" t="s">
         <v>248</v>
       </c>
-      <c r="C2" s="322"/>
-      <c r="D2" s="331"/>
-      <c r="E2" s="332"/>
-      <c r="F2" s="332"/>
-      <c r="G2" s="332"/>
-      <c r="H2" s="332"/>
-      <c r="I2" s="332"/>
-      <c r="J2" s="333"/>
+      <c r="C2" s="324"/>
+      <c r="D2" s="333"/>
+      <c r="E2" s="334"/>
+      <c r="F2" s="334"/>
+      <c r="G2" s="334"/>
+      <c r="H2" s="334"/>
+      <c r="I2" s="334"/>
+      <c r="J2" s="335"/>
     </row>
     <row r="3" spans="1:10" ht="21" customHeight="1">
       <c r="A3" s="94"/>
-      <c r="B3" s="322" t="s">
+      <c r="B3" s="324" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="322"/>
-      <c r="D3" s="324"/>
-      <c r="E3" s="325"/>
-      <c r="F3" s="334"/>
-      <c r="G3" s="335" t="s">
+      <c r="C3" s="324"/>
+      <c r="D3" s="326"/>
+      <c r="E3" s="327"/>
+      <c r="F3" s="336"/>
+      <c r="G3" s="337" t="s">
         <v>10</v>
       </c>
-      <c r="H3" s="336"/>
-      <c r="I3" s="337"/>
-      <c r="J3" s="317"/>
+      <c r="H3" s="338"/>
+      <c r="I3" s="339"/>
+      <c r="J3" s="319"/>
     </row>
     <row r="4" spans="1:10" ht="21" customHeight="1">
       <c r="A4" s="94"/>
-      <c r="B4" s="322" t="s">
+      <c r="B4" s="324" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="322"/>
-      <c r="D4" s="324"/>
-      <c r="E4" s="325"/>
-      <c r="F4" s="325"/>
-      <c r="G4" s="325"/>
-      <c r="H4" s="325"/>
-      <c r="I4" s="325"/>
-      <c r="J4" s="326"/>
+      <c r="C4" s="324"/>
+      <c r="D4" s="326"/>
+      <c r="E4" s="327"/>
+      <c r="F4" s="327"/>
+      <c r="G4" s="327"/>
+      <c r="H4" s="327"/>
+      <c r="I4" s="327"/>
+      <c r="J4" s="328"/>
     </row>
     <row r="5" spans="1:10" ht="21" customHeight="1">
       <c r="A5" s="95"/>
-      <c r="B5" s="322" t="s">
+      <c r="B5" s="324" t="s">
         <v>249</v>
       </c>
-      <c r="C5" s="322"/>
-      <c r="D5" s="310"/>
-      <c r="E5" s="311"/>
-      <c r="F5" s="311"/>
-      <c r="G5" s="311"/>
-      <c r="H5" s="311"/>
-      <c r="I5" s="311"/>
-      <c r="J5" s="312"/>
+      <c r="C5" s="324"/>
+      <c r="D5" s="312"/>
+      <c r="E5" s="313"/>
+      <c r="F5" s="313"/>
+      <c r="G5" s="313"/>
+      <c r="H5" s="313"/>
+      <c r="I5" s="313"/>
+      <c r="J5" s="314"/>
     </row>
     <row r="6" spans="1:10" ht="21" customHeight="1">
       <c r="A6" s="95"/>
-      <c r="B6" s="322" t="s">
+      <c r="B6" s="324" t="s">
         <v>250</v>
       </c>
-      <c r="C6" s="322"/>
-      <c r="D6" s="310"/>
-      <c r="E6" s="311"/>
-      <c r="F6" s="311"/>
-      <c r="G6" s="311"/>
-      <c r="H6" s="311"/>
-      <c r="I6" s="311"/>
-      <c r="J6" s="312"/>
+      <c r="C6" s="324"/>
+      <c r="D6" s="312"/>
+      <c r="E6" s="313"/>
+      <c r="F6" s="313"/>
+      <c r="G6" s="313"/>
+      <c r="H6" s="313"/>
+      <c r="I6" s="313"/>
+      <c r="J6" s="314"/>
     </row>
     <row r="7" spans="1:10" ht="21" customHeight="1">
       <c r="A7" s="95"/>
-      <c r="B7" s="322" t="s">
+      <c r="B7" s="324" t="s">
         <v>251</v>
       </c>
-      <c r="C7" s="322"/>
-      <c r="D7" s="327"/>
-      <c r="E7" s="328"/>
-      <c r="F7" s="328"/>
-      <c r="G7" s="328"/>
-      <c r="H7" s="328"/>
-      <c r="I7" s="328"/>
-      <c r="J7" s="329"/>
+      <c r="C7" s="324"/>
+      <c r="D7" s="329"/>
+      <c r="E7" s="330"/>
+      <c r="F7" s="330"/>
+      <c r="G7" s="330"/>
+      <c r="H7" s="330"/>
+      <c r="I7" s="330"/>
+      <c r="J7" s="331"/>
     </row>
     <row r="8" spans="1:10" ht="21" customHeight="1">
       <c r="A8" s="95"/>
-      <c r="B8" s="322" t="s">
+      <c r="B8" s="324" t="s">
         <v>252</v>
       </c>
-      <c r="C8" s="322"/>
-      <c r="D8" s="327"/>
-      <c r="E8" s="328"/>
-      <c r="F8" s="328"/>
-      <c r="G8" s="328"/>
-      <c r="H8" s="328"/>
-      <c r="I8" s="328"/>
-      <c r="J8" s="329"/>
+      <c r="C8" s="324"/>
+      <c r="D8" s="329"/>
+      <c r="E8" s="330"/>
+      <c r="F8" s="330"/>
+      <c r="G8" s="330"/>
+      <c r="H8" s="330"/>
+      <c r="I8" s="330"/>
+      <c r="J8" s="331"/>
     </row>
     <row r="9" spans="1:10" ht="21" customHeight="1">
       <c r="A9" s="96">
         <v>24</v>
       </c>
-      <c r="B9" s="323" t="s">
+      <c r="B9" s="325" t="s">
         <v>253</v>
       </c>
-      <c r="C9" s="323"/>
-      <c r="D9" s="310"/>
-      <c r="E9" s="311"/>
-      <c r="F9" s="311"/>
-      <c r="G9" s="311"/>
-      <c r="H9" s="311"/>
-      <c r="I9" s="311"/>
-      <c r="J9" s="312"/>
+      <c r="C9" s="325"/>
+      <c r="D9" s="312"/>
+      <c r="E9" s="313"/>
+      <c r="F9" s="313"/>
+      <c r="G9" s="313"/>
+      <c r="H9" s="313"/>
+      <c r="I9" s="313"/>
+      <c r="J9" s="314"/>
     </row>
     <row r="10" spans="1:10" ht="21" customHeight="1">
       <c r="A10" s="94"/>
-      <c r="B10" s="322" t="s">
+      <c r="B10" s="324" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="322"/>
-      <c r="D10" s="310"/>
-      <c r="E10" s="311"/>
-      <c r="F10" s="313"/>
-      <c r="G10" s="314" t="s">
+      <c r="C10" s="324"/>
+      <c r="D10" s="312"/>
+      <c r="E10" s="313"/>
+      <c r="F10" s="315"/>
+      <c r="G10" s="316" t="s">
         <v>10</v>
       </c>
-      <c r="H10" s="315"/>
-      <c r="I10" s="316"/>
-      <c r="J10" s="317"/>
+      <c r="H10" s="317"/>
+      <c r="I10" s="318"/>
+      <c r="J10" s="319"/>
     </row>
     <row r="11" spans="1:10" ht="21" customHeight="1">
       <c r="A11" s="94"/>
-      <c r="B11" s="322" t="s">
+      <c r="B11" s="324" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="322"/>
-      <c r="D11" s="318"/>
-      <c r="E11" s="311"/>
-      <c r="F11" s="311"/>
-      <c r="G11" s="311"/>
-      <c r="H11" s="311"/>
-      <c r="I11" s="311"/>
-      <c r="J11" s="312"/>
+      <c r="C11" s="324"/>
+      <c r="D11" s="320"/>
+      <c r="E11" s="313"/>
+      <c r="F11" s="313"/>
+      <c r="G11" s="313"/>
+      <c r="H11" s="313"/>
+      <c r="I11" s="313"/>
+      <c r="J11" s="314"/>
     </row>
     <row r="12" spans="1:10" ht="21" customHeight="1">
       <c r="A12" s="97">
         <v>25</v>
       </c>
-      <c r="B12" s="319" t="s">
+      <c r="B12" s="321" t="s">
         <v>254</v>
       </c>
-      <c r="C12" s="320"/>
-      <c r="D12" s="320"/>
-      <c r="E12" s="320"/>
-      <c r="F12" s="320"/>
-      <c r="G12" s="320"/>
-      <c r="H12" s="320"/>
-      <c r="I12" s="320"/>
-      <c r="J12" s="321"/>
+      <c r="C12" s="322"/>
+      <c r="D12" s="322"/>
+      <c r="E12" s="322"/>
+      <c r="F12" s="322"/>
+      <c r="G12" s="322"/>
+      <c r="H12" s="322"/>
+      <c r="I12" s="322"/>
+      <c r="J12" s="323"/>
     </row>
     <row r="13" spans="1:10" ht="21" customHeight="1">
       <c r="A13" s="94"/>
-      <c r="B13" s="322" t="s">
+      <c r="B13" s="324" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="322"/>
-      <c r="D13" s="310"/>
-      <c r="E13" s="311"/>
-      <c r="F13" s="311"/>
-      <c r="G13" s="311"/>
-      <c r="H13" s="311"/>
-      <c r="I13" s="311"/>
-      <c r="J13" s="312"/>
+      <c r="C13" s="324"/>
+      <c r="D13" s="312"/>
+      <c r="E13" s="313"/>
+      <c r="F13" s="313"/>
+      <c r="G13" s="313"/>
+      <c r="H13" s="313"/>
+      <c r="I13" s="313"/>
+      <c r="J13" s="314"/>
     </row>
     <row r="14" spans="1:10" ht="21" customHeight="1">
       <c r="A14" s="94"/>
-      <c r="B14" s="322" t="s">
+      <c r="B14" s="324" t="s">
         <v>9</v>
       </c>
-      <c r="C14" s="322"/>
-      <c r="D14" s="310"/>
-      <c r="E14" s="311"/>
-      <c r="F14" s="311"/>
-      <c r="G14" s="311"/>
-      <c r="H14" s="311"/>
-      <c r="I14" s="311"/>
-      <c r="J14" s="312"/>
+      <c r="C14" s="324"/>
+      <c r="D14" s="312"/>
+      <c r="E14" s="313"/>
+      <c r="F14" s="313"/>
+      <c r="G14" s="313"/>
+      <c r="H14" s="313"/>
+      <c r="I14" s="313"/>
+      <c r="J14" s="314"/>
     </row>
     <row r="15" spans="1:10" ht="21" customHeight="1" thickBot="1">
       <c r="A15" s="98"/>
-      <c r="B15" s="322" t="s">
+      <c r="B15" s="324" t="s">
         <v>13</v>
       </c>
-      <c r="C15" s="322"/>
-      <c r="D15" s="310"/>
-      <c r="E15" s="311"/>
-      <c r="F15" s="311"/>
-      <c r="G15" s="311"/>
-      <c r="H15" s="311"/>
-      <c r="I15" s="311"/>
-      <c r="J15" s="312"/>
+      <c r="C15" s="324"/>
+      <c r="D15" s="312"/>
+      <c r="E15" s="313"/>
+      <c r="F15" s="313"/>
+      <c r="G15" s="313"/>
+      <c r="H15" s="313"/>
+      <c r="I15" s="313"/>
+      <c r="J15" s="314"/>
     </row>
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="94KVciG4kdECMCBRaZ/kGUPIuUdTIjG67RnmSldA6WYOzuQmRnZSJRxdUi03GpwtwoEXd0J15wJilUTAVO1QkA==" saltValue="4px6JZ8PPWxSqTy644m1tg==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
@@ -18329,14 +18360,14 @@
       <c r="F1" s="120"/>
       <c r="G1" s="121"/>
       <c r="H1" s="119"/>
-      <c r="I1" s="338" t="s">
+      <c r="I1" s="340" t="s">
         <v>258</v>
       </c>
-      <c r="J1" s="338"/>
-      <c r="K1" s="338"/>
-      <c r="L1" s="338"/>
-      <c r="M1" s="338"/>
-      <c r="N1" s="338"/>
+      <c r="J1" s="340"/>
+      <c r="K1" s="340"/>
+      <c r="L1" s="340"/>
+      <c r="M1" s="340"/>
+      <c r="N1" s="340"/>
     </row>
     <row r="2" spans="1:14" ht="18" customHeight="1">
       <c r="A2" s="107" t="s">
@@ -18344,17 +18375,17 @@
       </c>
       <c r="B2" s="108"/>
       <c r="C2" s="108"/>
-      <c r="D2" s="345" t="s">
+      <c r="D2" s="347" t="s">
         <v>259</v>
       </c>
-      <c r="E2" s="346"/>
-      <c r="F2" s="339" t="s">
+      <c r="E2" s="348"/>
+      <c r="F2" s="341" t="s">
         <v>260</v>
       </c>
-      <c r="G2" s="339" t="s">
+      <c r="G2" s="341" t="s">
         <v>323</v>
       </c>
-      <c r="H2" s="342" t="s">
+      <c r="H2" s="344" t="s">
         <v>261</v>
       </c>
     </row>
@@ -18368,11 +18399,11 @@
       <c r="C3" s="110" t="s">
         <v>263</v>
       </c>
-      <c r="D3" s="347"/>
-      <c r="E3" s="348"/>
-      <c r="F3" s="340"/>
-      <c r="G3" s="340"/>
-      <c r="H3" s="343"/>
+      <c r="D3" s="349"/>
+      <c r="E3" s="350"/>
+      <c r="F3" s="342"/>
+      <c r="G3" s="342"/>
+      <c r="H3" s="345"/>
     </row>
     <row r="4" spans="1:14" ht="18" customHeight="1">
       <c r="A4" s="111"/>
@@ -18384,9 +18415,9 @@
       <c r="E4" s="115" t="s">
         <v>265</v>
       </c>
-      <c r="F4" s="341"/>
-      <c r="G4" s="341"/>
-      <c r="H4" s="344"/>
+      <c r="F4" s="343"/>
+      <c r="G4" s="343"/>
+      <c r="H4" s="346"/>
     </row>
     <row r="5" spans="1:14">
       <c r="A5" s="122"/>
@@ -18563,13 +18594,13 @@
       <c r="D1" s="133"/>
       <c r="E1" s="133"/>
       <c r="F1" s="133"/>
-      <c r="G1" s="351"/>
-      <c r="H1" s="351"/>
-      <c r="I1" s="351"/>
-      <c r="J1" s="351"/>
-      <c r="K1" s="351"/>
-      <c r="L1" s="351"/>
-      <c r="M1" s="351"/>
+      <c r="G1" s="353"/>
+      <c r="H1" s="353"/>
+      <c r="I1" s="353"/>
+      <c r="J1" s="353"/>
+      <c r="K1" s="353"/>
+      <c r="L1" s="353"/>
+      <c r="M1" s="353"/>
     </row>
     <row r="2" spans="1:14" ht="31.5" customHeight="1">
       <c r="A2" s="134"/>
@@ -18593,10 +18624,10 @@
       <c r="D3" s="141" t="s">
         <v>268</v>
       </c>
-      <c r="E3" s="349" t="s">
+      <c r="E3" s="351" t="s">
         <v>269</v>
       </c>
-      <c r="F3" s="350"/>
+      <c r="F3" s="352"/>
       <c r="N3" s="103"/>
     </row>
     <row r="4" spans="1:14" ht="31.5" customHeight="1">
@@ -19588,63 +19619,63 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30.75" customHeight="1">
-      <c r="A1" s="352" t="s">
+      <c r="A1" s="354" t="s">
         <v>271</v>
       </c>
-      <c r="B1" s="353"/>
-      <c r="C1" s="353"/>
-      <c r="D1" s="353"/>
-      <c r="E1" s="353"/>
-      <c r="F1" s="353"/>
-      <c r="G1" s="353"/>
-      <c r="H1" s="354"/>
+      <c r="B1" s="355"/>
+      <c r="C1" s="355"/>
+      <c r="D1" s="355"/>
+      <c r="E1" s="355"/>
+      <c r="F1" s="355"/>
+      <c r="G1" s="355"/>
+      <c r="H1" s="356"/>
     </row>
     <row r="2" spans="1:14" ht="30.75" customHeight="1" thickBot="1">
-      <c r="A2" s="355" t="s">
+      <c r="A2" s="357" t="s">
         <v>272</v>
       </c>
-      <c r="B2" s="356"/>
-      <c r="C2" s="356"/>
-      <c r="D2" s="356"/>
-      <c r="E2" s="356"/>
-      <c r="F2" s="356"/>
-      <c r="G2" s="356"/>
-      <c r="H2" s="357"/>
+      <c r="B2" s="358"/>
+      <c r="C2" s="358"/>
+      <c r="D2" s="358"/>
+      <c r="E2" s="358"/>
+      <c r="F2" s="358"/>
+      <c r="G2" s="358"/>
+      <c r="H2" s="359"/>
     </row>
     <row r="3" spans="1:14" ht="30.75" customHeight="1">
-      <c r="A3" s="367" t="s">
+      <c r="A3" s="369" t="s">
         <v>326</v>
       </c>
-      <c r="B3" s="368"/>
-      <c r="C3" s="358" t="s">
+      <c r="B3" s="370"/>
+      <c r="C3" s="360" t="s">
         <v>273</v>
       </c>
-      <c r="D3" s="361" t="s">
+      <c r="D3" s="363" t="s">
         <v>274</v>
       </c>
-      <c r="E3" s="361" t="s">
+      <c r="E3" s="363" t="s">
         <v>275</v>
       </c>
-      <c r="F3" s="361" t="s">
+      <c r="F3" s="363" t="s">
         <v>276</v>
       </c>
-      <c r="G3" s="339" t="s">
+      <c r="G3" s="341" t="s">
         <v>277</v>
       </c>
-      <c r="H3" s="364" t="s">
+      <c r="H3" s="366" t="s">
         <v>322</v>
       </c>
       <c r="N3" s="152"/>
     </row>
     <row r="4" spans="1:14" ht="30.75" customHeight="1">
-      <c r="A4" s="369"/>
-      <c r="B4" s="370"/>
-      <c r="C4" s="359"/>
-      <c r="D4" s="362"/>
-      <c r="E4" s="362"/>
-      <c r="F4" s="362"/>
-      <c r="G4" s="340"/>
-      <c r="H4" s="365"/>
+      <c r="A4" s="371"/>
+      <c r="B4" s="372"/>
+      <c r="C4" s="361"/>
+      <c r="D4" s="364"/>
+      <c r="E4" s="364"/>
+      <c r="F4" s="364"/>
+      <c r="G4" s="342"/>
+      <c r="H4" s="367"/>
       <c r="N4" s="152"/>
     </row>
     <row r="5" spans="1:14" ht="30.75" customHeight="1">
@@ -19654,12 +19685,12 @@
       <c r="B5" s="146" t="s">
         <v>265</v>
       </c>
-      <c r="C5" s="360"/>
-      <c r="D5" s="363"/>
-      <c r="E5" s="363"/>
-      <c r="F5" s="363"/>
-      <c r="G5" s="341"/>
-      <c r="H5" s="366"/>
+      <c r="C5" s="362"/>
+      <c r="D5" s="365"/>
+      <c r="E5" s="365"/>
+      <c r="F5" s="365"/>
+      <c r="G5" s="343"/>
+      <c r="H5" s="368"/>
       <c r="N5" s="152"/>
     </row>
     <row r="6" spans="1:14">
@@ -19971,17 +20002,17 @@
       <c r="Q1" s="142"/>
     </row>
     <row r="2" spans="1:17" ht="23.25" customHeight="1">
-      <c r="A2" s="371" t="s">
+      <c r="A2" s="373" t="s">
         <v>279</v>
       </c>
-      <c r="B2" s="358" t="s">
+      <c r="B2" s="360" t="s">
         <v>327</v>
       </c>
-      <c r="C2" s="377"/>
-      <c r="D2" s="361" t="s">
+      <c r="C2" s="379"/>
+      <c r="D2" s="363" t="s">
         <v>280</v>
       </c>
-      <c r="E2" s="374" t="s">
+      <c r="E2" s="376" t="s">
         <v>281</v>
       </c>
       <c r="F2" s="158"/>
@@ -19998,11 +20029,11 @@
       <c r="Q2" s="142"/>
     </row>
     <row r="3" spans="1:17" ht="23.25" customHeight="1">
-      <c r="A3" s="372"/>
-      <c r="B3" s="359"/>
-      <c r="C3" s="378"/>
-      <c r="D3" s="362"/>
-      <c r="E3" s="375"/>
+      <c r="A3" s="374"/>
+      <c r="B3" s="361"/>
+      <c r="C3" s="380"/>
+      <c r="D3" s="364"/>
+      <c r="E3" s="377"/>
       <c r="F3" s="158"/>
       <c r="G3" s="142"/>
       <c r="H3" s="142"/>
@@ -20017,15 +20048,15 @@
       <c r="Q3" s="142"/>
     </row>
     <row r="4" spans="1:17" ht="23.25" customHeight="1">
-      <c r="A4" s="373"/>
+      <c r="A4" s="375"/>
       <c r="B4" s="146" t="s">
         <v>264</v>
       </c>
       <c r="C4" s="146" t="s">
         <v>265</v>
       </c>
-      <c r="D4" s="363"/>
-      <c r="E4" s="376"/>
+      <c r="D4" s="365"/>
+      <c r="E4" s="378"/>
       <c r="F4" s="158"/>
       <c r="G4" s="142"/>
       <c r="H4" s="142"/>
@@ -20514,62 +20545,62 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30.75" customHeight="1">
-      <c r="A1" s="379" t="s">
+      <c r="A1" s="381" t="s">
         <v>282</v>
       </c>
-      <c r="B1" s="380"/>
-      <c r="C1" s="380"/>
-      <c r="D1" s="380"/>
-      <c r="E1" s="380"/>
-      <c r="F1" s="381"/>
+      <c r="B1" s="382"/>
+      <c r="C1" s="382"/>
+      <c r="D1" s="382"/>
+      <c r="E1" s="382"/>
+      <c r="F1" s="383"/>
     </row>
     <row r="2" spans="1:8" ht="30.75" customHeight="1">
-      <c r="A2" s="382" t="s">
+      <c r="A2" s="384" t="s">
         <v>283</v>
       </c>
-      <c r="B2" s="383"/>
-      <c r="C2" s="383"/>
-      <c r="D2" s="383"/>
-      <c r="E2" s="383"/>
-      <c r="F2" s="384"/>
+      <c r="B2" s="385"/>
+      <c r="C2" s="385"/>
+      <c r="D2" s="385"/>
+      <c r="E2" s="385"/>
+      <c r="F2" s="386"/>
     </row>
     <row r="3" spans="1:8" ht="30.75" customHeight="1">
-      <c r="A3" s="385" t="s">
+      <c r="A3" s="387" t="s">
         <v>284</v>
       </c>
-      <c r="B3" s="390" t="s">
+      <c r="B3" s="392" t="s">
         <v>328</v>
       </c>
-      <c r="C3" s="391"/>
-      <c r="D3" s="387" t="s">
+      <c r="C3" s="393"/>
+      <c r="D3" s="389" t="s">
         <v>280</v>
       </c>
-      <c r="E3" s="362" t="s">
+      <c r="E3" s="364" t="s">
         <v>285</v>
       </c>
-      <c r="F3" s="389" t="s">
+      <c r="F3" s="391" t="s">
         <v>286</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="30.75" customHeight="1">
-      <c r="A4" s="386"/>
-      <c r="B4" s="359"/>
-      <c r="C4" s="392"/>
-      <c r="D4" s="387"/>
-      <c r="E4" s="362"/>
-      <c r="F4" s="375"/>
+      <c r="A4" s="388"/>
+      <c r="B4" s="361"/>
+      <c r="C4" s="394"/>
+      <c r="D4" s="389"/>
+      <c r="E4" s="364"/>
+      <c r="F4" s="377"/>
     </row>
     <row r="5" spans="1:8" ht="30.75" customHeight="1">
-      <c r="A5" s="369"/>
+      <c r="A5" s="371"/>
       <c r="B5" s="146" t="s">
         <v>264</v>
       </c>
       <c r="C5" s="146" t="s">
         <v>265</v>
       </c>
-      <c r="D5" s="388"/>
-      <c r="E5" s="363"/>
-      <c r="F5" s="376"/>
+      <c r="D5" s="390"/>
+      <c r="E5" s="365"/>
+      <c r="F5" s="378"/>
     </row>
     <row r="6" spans="1:8" ht="18.75" customHeight="1">
       <c r="A6" s="161"/>
@@ -20771,11 +20802,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="27.75" customHeight="1">
-      <c r="A1" s="393" t="s">
+      <c r="A1" s="395" t="s">
         <v>287</v>
       </c>
-      <c r="B1" s="394"/>
-      <c r="C1" s="395"/>
+      <c r="B1" s="396"/>
+      <c r="C1" s="397"/>
     </row>
     <row r="2" spans="1:13" ht="38.25" customHeight="1">
       <c r="A2" s="163" t="s">

</xml_diff>